<commit_message>
Corrigir títulos e cargas horárias verificadas no Coursera
</commit_message>
<xml_diff>
--- a/ACG_UNIFENAS_Medicina.xlsx
+++ b/ACG_UNIFENAS_Medicina.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R468e890910824663"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regras UNIFENAS" sheetId="2" r:id="Ra7d04fb282a24b17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Certificados" sheetId="3" r:id="R219b2c340da94971"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluídos" sheetId="4" r:id="R825f1c0c07834f4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pendências" sheetId="5" r:id="R02d4692ebe774030"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rbcb49d509f77490b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regras UNIFENAS" sheetId="2" r:id="R27aab66ab4c64650"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Certificados" sheetId="3" r:id="Rcf6dbe21f640464a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluídos" sheetId="4" r:id="R17671312f80c41f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pendências" sheetId="5" r:id="R4a2acac1b43f46e1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -466,7 +466,7 @@
       </x:c>
       <x:c r="B6" s="16" t="n">
         <x:f>SUM('Certificados'!$J$2:$J$389)</x:f>
-        <x:v>1087.5</x:v>
+        <x:v>2084.5</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -475,7 +475,7 @@
       </x:c>
       <x:c r="B7" s="16" t="n">
         <x:f>SUM('Certificados'!$K$2:$K$389)</x:f>
-        <x:v>1087.5</x:v>
+        <x:v>2084.5</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -484,7 +484,7 @@
       </x:c>
       <x:c r="B8" s="16" t="n">
         <x:f>B3-B7</x:f>
-        <x:v>-637.5</x:v>
+        <x:v>-1634.5</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -519,11 +519,11 @@
       </x:c>
       <x:c r="C12" s="30" t="n">
         <x:f>SUMIF('Certificados'!$G$2:$G$389,A12,'Certificados'!$J$2:$J$389)</x:f>
-        <x:v>413.25</x:v>
+        <x:v>1410.25</x:v>
       </x:c>
       <x:c r="D12" s="30" t="n">
         <x:f>SUMIF('Certificados'!$G$2:$G$389,A12,'Certificados'!$K$2:$K$389)</x:f>
-        <x:v>413.25</x:v>
+        <x:v>1410.25</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2012,10 +2012,10 @@
         <x:v>BSI-Coursera ISO 42001 Readiness Specialization Certificate K99N55L2EZNG.pdf</x:v>
       </x:c>
       <x:c r="C26" s="32" t="str">
-        <x:v>BSI</x:v>
+        <x:v>British Standards Institution (BSI)</x:v>
       </x:c>
       <x:c r="D26" s="32" t="str">
-        <x:v>BSI-Coursera ISO 42001 Readiness Specialization Certificate K99N55L2EZNG</x:v>
+        <x:v>AI Governance &amp; ISO 42001 Readiness for GRC, Audit, &amp; Legal</x:v>
       </x:c>
       <x:c r="E26" s="32" t="str">
         <x:v>5 C o u r s e s I S O / I E C 2 2 9 8 9 : 2 0 2 3 A n I n t r o d u c t i o n t o t h e F u n d a m e n t a l s o f A I A I S y s t e m I m p a c t A s s e s s m e n t G u i d a n c e A I M a n a g e m e n t E s s e n t i a l s : I n t e g r a t i n g I S O 4 2 0 0 1 &amp; I S O 2 3 8 9 4 U n d e r s t a n d i n g t h e F o u n d a t i o n s o f t h e E U A I A c t A p p r o a c h e s t o E s t a b l i s h T r u s t i n A I S y s t e m s H e c t o r N e m o t o , B S I G l o b a l T r a i n i n g D </x:v>
@@ -2030,11 +2030,17 @@
       <x:c r="I26" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J26" s="33"/>
-      <x:c r="K26" s="33"/>
-      <x:c r="L26" s="33"/>
+      <x:c r="J26" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="K26" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="L26" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
       <x:c r="M26" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/K99N55L2EZNG; estimativa derivada do tempo exibido: 1 meses com 10 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -2045,10 +2051,10 @@
         <x:v>BSI-Coursera_AIMS Essentials Certificate_7M8MXVWELB5L.pdf</x:v>
       </x:c>
       <x:c r="C27" s="32" t="str">
-        <x:v>BSI</x:v>
+        <x:v>British Standards Institution (BSI)</x:v>
       </x:c>
       <x:c r="D27" s="32" t="str">
-        <x:v>BSI-Coursera_AIMS Essentials Certificate_7M8MXVWELB5L</x:v>
+        <x:v>AI Management Essentials: Integrating ISO 42001 &amp; ISO 23894</x:v>
       </x:c>
       <x:c r="E27" s="32" t="str">
         <x:v>A u g 1 5 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o A I M a n a g e m e n t E s s e n t i a l s : I n t e g r a t i n g I S O 4 2 0 0 1 &amp; I S O 2 3 8 9 4 a n o n l i n e c o u r s e a u t h o r i z e d b y B r i t i s h S t a n d a r d s I n s t i t u t i o n a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d H e c t o r N e m o t o B S I G l o b a l T r a i n i n g D i r e c t o r V e r i f y a t : h t t p s : / / c o u r s e r a . o r g </x:v>
@@ -2063,11 +2069,17 @@
       <x:c r="I27" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J27" s="33"/>
-      <x:c r="K27" s="33"/>
-      <x:c r="L27" s="33"/>
+      <x:c r="J27" s="33" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K27" s="33" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="L27" s="33" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="M27" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/7M8MXVWELB5L</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -2078,10 +2090,10 @@
         <x:v>BSI-Coursera_AISIA_Certificate JMK7JAW5O7R9.pdf</x:v>
       </x:c>
       <x:c r="C28" s="32" t="str">
-        <x:v>BSI</x:v>
+        <x:v>British Standards Institution (BSI)</x:v>
       </x:c>
       <x:c r="D28" s="32" t="str">
-        <x:v>BSI-Coursera_AISIA_Certificate JMK7JAW5O7R9</x:v>
+        <x:v>AI System Impact Assessment Guidance</x:v>
       </x:c>
       <x:c r="E28" s="32" t="str">
         <x:v>A u g 1 4 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o A I S y s t e m I m p a c t A s s e s s m e n t G u i d a n c e a n o n l i n e c o u r s e a u t h o r i z e d b y B r i t i s h S t a n d a r d s I n s t i t u t i o n a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d H e c t o r N e m o t o B S I G l o b a l T r a i n i n g D i r e c t o r V e r i f y a t : h t t p s : / / c o u r s e r a . o r g / v e r i f y / J M K 7 J A W 5 O 7 R </x:v>
@@ -2096,11 +2108,17 @@
       <x:c r="I28" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J28" s="33"/>
-      <x:c r="K28" s="33"/>
-      <x:c r="L28" s="33"/>
+      <x:c r="J28" s="33" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K28" s="33" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L28" s="33" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="M28" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/JMK7JAW5O7R9</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -2111,10 +2129,10 @@
         <x:v>BSI-Coursera_EU AI Act_CertificateE0NA98PI4EVM.pdf</x:v>
       </x:c>
       <x:c r="C29" s="32" t="str">
-        <x:v>BSI</x:v>
+        <x:v>British Standards Institution (BSI)</x:v>
       </x:c>
       <x:c r="D29" s="32" t="str">
-        <x:v>BSI-Coursera_EU AI Act_CertificateE0NA98PI4EVM</x:v>
+        <x:v>Understanding the Foundations of the EU AI Act</x:v>
       </x:c>
       <x:c r="E29" s="32" t="str">
         <x:v>A u g 1 4 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o U n d e r s t a n d i n g t h e F o u n d a t i o n s o f t h e E U A I A c t a n o n l i n e c o u r s e a u t h o r i z e d b y B r i t i s h S t a n d a r d s I n s t i t u t i o n a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d H e c t o r N e m o t o B S I G l o b a l T r a i n i n g D i r e c t o r V e r i f y a t : h t t p s : / / c o u r s e r a . o r g / v e r i f y / E 0 N A </x:v>
@@ -2129,11 +2147,17 @@
       <x:c r="I29" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J29" s="33"/>
-      <x:c r="K29" s="33"/>
-      <x:c r="L29" s="33"/>
+      <x:c r="J29" s="33" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K29" s="33" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L29" s="33" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="M29" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/E0NA98PI4EVM</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -2144,10 +2168,10 @@
         <x:v>BSI-Coursera_Intro ISO 22989 Certificate_3HLETUDTZKS9.pdf</x:v>
       </x:c>
       <x:c r="C30" s="32" t="str">
-        <x:v>BSI</x:v>
+        <x:v>British Standards Institution (BSI)</x:v>
       </x:c>
       <x:c r="D30" s="32" t="str">
-        <x:v>BSI-Coursera_Intro ISO 22989 Certificate_3HLETUDTZKS9</x:v>
+        <x:v>ISO/IEC 22989:2023 An Introduction to the Fundamentals of AI</x:v>
       </x:c>
       <x:c r="E30" s="32" t="str">
         <x:v>A u g 1 3 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o I S O / I E C 2 2 9 8 9 : 2 0 2 3 A n I n t r o d u c t i o n t o t h e F u n d a m e n t a l s o f A I a n o n l i n e c o u r s e a u t h o r i z e d b y B r i t i s h S t a n d a r d s I n s t i t u t i o n a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d H e c t o r N e m o t o B S I G l o b a l T r a i n i n g D i r e c t o r V e r i f y a t : h t t p s : / / c o u r s e r a . o r </x:v>
@@ -2163,15 +2187,17 @@
         <x:v>Extraído do documento</x:v>
       </x:c>
       <x:c r="J30" s="33" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="K30" s="33" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L30" s="33" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="M30" s="32" t="str"/>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M30" s="32" t="str">
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/3HLETUDTZKS9</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="32" t="n">
@@ -3278,10 +3304,10 @@
         <x:v>Certificado JHU+Coursera SVWCQ560O1OU - Revenue Cycle, Billing and Coding.jpg</x:v>
       </x:c>
       <x:c r="C64" s="32" t="str">
-        <x:v>Certificado JHU+Coursera SVWCQ560O1OU</x:v>
+        <x:v>Johns Hopkins University</x:v>
       </x:c>
       <x:c r="D64" s="32" t="str">
-        <x:v>Certificado JHU+Coursera SVWCQ560O1OU - Revenue Cycle, Billing and Coding</x:v>
+        <x:v>Revenue Cycle, Billing, and Coding</x:v>
       </x:c>
       <x:c r="E64" s="32" t="str"/>
       <x:c r="F64" s="32" t="str"/>
@@ -3294,11 +3320,17 @@
       <x:c r="I64" s="32" t="str">
         <x:v>Sem texto extraível — revisão manual</x:v>
       </x:c>
-      <x:c r="J64" s="33"/>
-      <x:c r="K64" s="33"/>
-      <x:c r="L64" s="33"/>
+      <x:c r="J64" s="33" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K64" s="33" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="L64" s="33" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="M64" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/SVWCQ560O1OU</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -3309,10 +3341,10 @@
         <x:v>Certificado JHU+Coursera SVWCQ560O1OU - Revenue Cycle, Billing and Coding.pdf</x:v>
       </x:c>
       <x:c r="C65" s="32" t="str">
-        <x:v>Certificado JHU+Coursera SVWCQ560O1OU</x:v>
+        <x:v>Johns Hopkins University</x:v>
       </x:c>
       <x:c r="D65" s="32" t="str">
-        <x:v>Certificado JHU+Coursera SVWCQ560O1OU - Revenue Cycle, Billing and Coding</x:v>
+        <x:v>Revenue Cycle, Billing, and Coding</x:v>
       </x:c>
       <x:c r="E65" s="32" t="str">
         <x:v>J u n 2 8 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o R e v e n u e C y c l e , B i l l i n g , a n d C o d i n g u m c u r s o o n - l i n e a u t o r i z a d o p e l a J o h n s H o p k i n s U n i v e r s i t y e m i n i s t r a d o a t r a v é s d a C o u r s e r a c o n c l u i u c o m s u c e s s o o P r o g r a m a d e c u r s o s i n t e g r a d o s M a u r a M c G u i r e , M D , C P C , F A C P E x e c u t i v e D i r e c t o r O J H P S t r a t e g i c L e a r n i n g C e n t </x:v>
@@ -3327,11 +3359,17 @@
       <x:c r="I65" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J65" s="33"/>
-      <x:c r="K65" s="33"/>
-      <x:c r="L65" s="33"/>
+      <x:c r="J65" s="33" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K65" s="33" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="L65" s="33" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="M65" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/SVWCQ560O1OU</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -3342,10 +3380,10 @@
         <x:v>Certificado Profissional JHU+Coursera P7PRAOBUU4L9 - JH Medical Office Manager (On-line).pdf</x:v>
       </x:c>
       <x:c r="C66" s="32" t="str">
-        <x:v>Certificado Profissional JHU+Coursera P7PRAOBUU4L9</x:v>
+        <x:v>Johns Hopkins University</x:v>
       </x:c>
       <x:c r="D66" s="32" t="str">
-        <x:v>Certificado Profissional JHU+Coursera P7PRAOBUU4L9 - JH Medical Office Manager (On-line)</x:v>
+        <x:v>Johns Hopkins Medical Office Manager</x:v>
       </x:c>
       <x:c r="E66" s="32" t="str">
         <x:v>Certificates Specialization Certificate Johns Hopkins Medical Office Manager Completed by Pedro Lamounier Sampaio June 28, 2026 Approximately 6 months at 3 hours a week to complete Pedro Lamounier Sampaio's account is veriﬁed. Coursera certiﬁestheir successful completion of Johns Hopkins University JohnsHopkins Medical Oﬃce Manager Specialization. Course Certiﬁcates Completed Introduction to Ambulatory Healthcare Management Human Resources Management Essentials Quality and Safety in Ambulatory H</x:v>
@@ -3361,16 +3399,16 @@
         <x:v>Extraído do documento</x:v>
       </x:c>
       <x:c r="J66" s="33" t="n">
-        <x:v>3</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="K66" s="33" t="n">
-        <x:v>3</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="L66" s="33" t="n">
-        <x:v>3</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="M66" s="32" t="str">
-        <x:v>https://www.coursera.org/account/accomplishments/professional-cert/P7PRAOBUU4L9</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/professional-cert/P7PRAOBUU4L9; estimativa derivada do tempo exibido: 6 meses com 3 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -3381,10 +3419,10 @@
         <x:v>Certificado Profissional JHU+Coursera P7PRAOBUU4L9 - JH Medical Office Manager.pdf</x:v>
       </x:c>
       <x:c r="C67" s="32" t="str">
-        <x:v>Certificado Profissional JHU+Coursera P7PRAOBUU4L9</x:v>
+        <x:v>Johns Hopkins University</x:v>
       </x:c>
       <x:c r="D67" s="32" t="str">
-        <x:v>Certificado Profissional JHU+Coursera P7PRAOBUU4L9 - JH Medical Office Manager</x:v>
+        <x:v>Johns Hopkins Medical Office Manager</x:v>
       </x:c>
       <x:c r="E67" s="32" t="str">
         <x:v>6 c u r s o s I n t r o d u c t i o n t o A m b u l a t o r y H e a l t h c a r e M a n a g e m e n t H u m a n R e s o u r c e s M a n a g e m e n t E s s e n t i a l s Q u a l i t y a n d S a f e t y i n A m b u l a t o r y H e a l t h c a r e M a n a g e m e n t H e a l t h c a r e D e l i v e r y f o r M e d i c a l P r a c t i c e M a n a g e r s D a t a a n d E l e c t r o n i c H e a l t h R e c o r d s R e v e n u e C y c l e , B i l l i n g , a n d C o d i n g M i c h e l l e J . C a m </x:v>
@@ -3399,11 +3437,17 @@
       <x:c r="I67" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J67" s="33"/>
-      <x:c r="K67" s="33"/>
-      <x:c r="L67" s="33"/>
+      <x:c r="J67" s="33" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="K67" s="33" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="L67" s="33" t="n">
+        <x:v>72</x:v>
+      </x:c>
       <x:c r="M67" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/professional-cert/P7PRAOBUU4L9; estimativa derivada do tempo exibido: 6 meses com 3 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -4225,10 +4269,10 @@
         <x:v>Coursera 4UIYZU51HN5L_JHU_Outbreaks and Epidemics.pdf</x:v>
       </x:c>
       <x:c r="C93" s="32" t="str">
-        <x:v>Coursera 4UIYZU51HN5L</x:v>
+        <x:v>Johns Hopkins University</x:v>
       </x:c>
       <x:c r="D93" s="32" t="str">
-        <x:v>Coursera 4UIYZU51HN5L_JHU_Outbreaks and Epidemics</x:v>
+        <x:v>Outbreaks and Epidemics</x:v>
       </x:c>
       <x:c r="E93" s="32" t="str">
         <x:v>J u l 1 9 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o O u t b r e a k s a n d E p i d e m i c s a n o n l i n e c o u r s e a u t h o r i z e d b y J o h n s H o p k i n s U n i v e r s i t y a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d J u s t i n L e s s l e r A s s o c i a t e P r o f e s s o r D e p a r t m e n t o f E p i d e m i o l o g y J o h n s H o p k i n s B l o o m b e r g S c h o o l o f P u b l i c H e a l t h V e r i f </x:v>
@@ -4244,15 +4288,17 @@
         <x:v>Extraído do documento</x:v>
       </x:c>
       <x:c r="J93" s="33" t="n">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="K93" s="33" t="n">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L93" s="33" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="M93" s="32" t="str"/>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M93" s="32" t="str">
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/4UIYZU51HN5L</x:v>
+      </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="32" t="n">
@@ -4261,11 +4307,9 @@
       <x:c r="B94" s="32" t="str">
         <x:v>Coursera 8BH1XC5QBHPD_Specialization_Epidemiology and PHP.pdf</x:v>
       </x:c>
-      <x:c r="C94" s="32" t="str">
-        <x:v>Coursera 8BH1XC5QBHPD</x:v>
-      </x:c>
+      <x:c r="C94" s="32" t="str"/>
       <x:c r="D94" s="32" t="str">
-        <x:v>Coursera 8BH1XC5QBHPD_Specialization_Epidemiology and PHP</x:v>
+        <x:v>Epidemiology in Public Health Practice</x:v>
       </x:c>
       <x:c r="E94" s="32" t="str">
         <x:v>5 C o u r s e s E s s e n t i a l E p i d e m i o l o g i c T o o l s f o r P u b l i c H e a l t h P r a c t i c e D a t a a n d H e a l t h I n d i c a t o r s i n P u b l i c H e a l t h P r a c t i c e S u r v e i l l a n c e S y s t e m s : T h e B u i l d i n g B l o c k s S u r v e i l l a n c e S y s t e m s : A n a l y s i s , D i s s e m i n a t i o n , a n d S p e c i a l S y s t e m s O u t b r e a k s a n d E p i d e m i c s K e r i A l t h o ﬀ , P h D J u l 1 9 , 2 0 2 6 P e d r o </x:v>
@@ -4280,11 +4324,17 @@
       <x:c r="I94" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J94" s="33"/>
-      <x:c r="K94" s="33"/>
-      <x:c r="L94" s="33"/>
+      <x:c r="J94" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="K94" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="L94" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
       <x:c r="M94" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/8BH1XC5QBHPD; estimativa derivada do tempo exibido: 1 meses com 10 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
@@ -4294,11 +4344,9 @@
       <x:c r="B95" s="32" t="str">
         <x:v>Coursera CUX1XMF3YS8E_Leading HC Q-S_GWU.pdf</x:v>
       </x:c>
-      <x:c r="C95" s="32" t="str">
-        <x:v>Coursera CUX1XMF3YS8E</x:v>
-      </x:c>
+      <x:c r="C95" s="32" t="str"/>
       <x:c r="D95" s="32" t="str">
-        <x:v>Coursera CUX1XMF3YS8E_Leading HC Q-S_GWU</x:v>
+        <x:v>Leading Healthcare Quality and Safety</x:v>
       </x:c>
       <x:c r="E95" s="32" t="str">
         <x:v>J u l 2 1 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o L e a d i n g H e a l t h c a r e Q u a l i t y a n d S a f e t y a n o n l i n e c o u r s e a u t h o r i z e d b y T h e G e o r g e W a s h i n g t o n U n i v e r s i t y a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d G r e g o r y P a w l s o n C l i n i c a l P r o f e s s o r o f M e d i c i n e a n d E x e c u t i v e C o a c h G W S c h o o l o f N u r s i n g J e a n J o h </x:v>
@@ -4313,11 +4361,17 @@
       <x:c r="I95" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J95" s="33"/>
-      <x:c r="K95" s="33"/>
-      <x:c r="L95" s="33"/>
+      <x:c r="J95" s="33" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="K95" s="33" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="L95" s="33" t="n">
+        <x:v>13</x:v>
+      </x:c>
       <x:c r="M95" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/CUX1XMF3YS8E</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
@@ -4328,10 +4382,10 @@
         <x:v>Coursera-Duke Certificate_TeleHealth KVF3XW2SP4BV.pdf</x:v>
       </x:c>
       <x:c r="C96" s="32" t="str">
-        <x:v>Coursera</x:v>
+        <x:v>Duke University</x:v>
       </x:c>
       <x:c r="D96" s="32" t="str">
-        <x:v>Coursera-Duke Certificate_TeleHealth KVF3XW2SP4BV</x:v>
+        <x:v>Telehealth Clinical Essentials</x:v>
       </x:c>
       <x:c r="E96" s="32" t="str">
         <x:v>J u l 2 5 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o T e l e h e a l t h C l i n i c a l E s s e n t i a l s a n o n l i n e c o u r s e a u t h o r i z e d b y D u k e U n i v e r s i t y a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d D a n i e l O s t r o v s k y A s s o c i a t e P r o f e s s o r P e d i a t r i c s K a t h l e e n W a i t e P r o f e s s o r o f M e d i c i n e D i v i s i o n o f G e n e r a l I n t e r n a l M e </x:v>
@@ -4346,11 +4400,17 @@
       <x:c r="I96" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J96" s="33"/>
-      <x:c r="K96" s="33"/>
-      <x:c r="L96" s="33"/>
+      <x:c r="J96" s="33" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K96" s="33" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L96" s="33" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="M96" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/KVF3XW2SP4BV</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
@@ -4361,10 +4421,10 @@
         <x:v>Coursera-ICL_Quality Improvement Specialization_Certificate 2RUAK3DPGYVQ.pdf</x:v>
       </x:c>
       <x:c r="C97" s="32" t="str">
-        <x:v>Coursera</x:v>
+        <x:v>Imperial College London</x:v>
       </x:c>
       <x:c r="D97" s="32" t="str">
-        <x:v>Coursera-ICL_Quality Improvement Specialization_Certificate 2RUAK3DPGYVQ</x:v>
+        <x:v>Quality Improvement in Healthcare</x:v>
       </x:c>
       <x:c r="E97" s="32" t="str">
         <x:v>3 C o u r s e s I n t r o d u c t i o n t o Q u a l i t y I m p r o v e m e n t i n H e a l t h c a r e U s i n g D a t a f o r H e a l t h c a r e I m p r o v e m e n t Q u a l i t y I m p r o v e m e n t f o r P o p u l a t i o n H e a l t h D r T h o m a s W o o d c o c k S e n i o r R e s e a r c h F e l l o w S c h o o l o f P u b l i c H e a l t h J u l 2 4 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o h a s s u c c e s s f u l l y c o m p l e t e d t h e o n l i n e S p e c i a l i </x:v>
@@ -4379,11 +4439,17 @@
       <x:c r="I97" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J97" s="33"/>
-      <x:c r="K97" s="33"/>
-      <x:c r="L97" s="33"/>
+      <x:c r="J97" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="K97" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="L97" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
       <x:c r="M97" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/2RUAK3DPGYVQ; estimativa derivada do tempo exibido: 1 meses com 10 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
@@ -4394,10 +4460,10 @@
         <x:v>Coursera.ICL_ONCEZO8V6040_Intro to Quality Improvement in HC.pdf</x:v>
       </x:c>
       <x:c r="C98" s="32" t="str">
-        <x:v>Coursera.ICL</x:v>
+        <x:v>Imperial College London</x:v>
       </x:c>
       <x:c r="D98" s="32" t="str">
-        <x:v>Coursera.ICL_ONCEZO8V6040_Intro to Quality Improvement in HC</x:v>
+        <x:v>Introduction to Quality Improvement in Healthcare</x:v>
       </x:c>
       <x:c r="E98" s="32" t="str">
         <x:v>J u l 2 2 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o I n t r o d u c t i o n t o Q u a l i t y I m p r o v e m e n t i n H e a l t h c a r e a n o n l i n e c o u r s e a u t h o r i z e d b y I m p e r i a l C o l l e g e L o n d o n a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d D r T h o m a s W o o d c o c k S e n i o r R e s e a r c h F e l l o w S c h o o l o f P u b l i c H e a l t h V e r i f y a t : h t t p s : / / c o u r s e </x:v>
@@ -4412,11 +4478,17 @@
       <x:c r="I98" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J98" s="33"/>
-      <x:c r="K98" s="33"/>
-      <x:c r="L98" s="33"/>
+      <x:c r="J98" s="33" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="K98" s="33" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="L98" s="33" t="n">
+        <x:v>21</x:v>
+      </x:c>
       <x:c r="M98" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/ONCEZO8V6040</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
@@ -4427,10 +4499,10 @@
         <x:v>Coursera_ICL_Certificate_Health Data Usage_V3XFWO53BYYT.pdf</x:v>
       </x:c>
       <x:c r="C99" s="32" t="str">
-        <x:v>Coursera</x:v>
+        <x:v>Imperial College London</x:v>
       </x:c>
       <x:c r="D99" s="32" t="str">
-        <x:v>Coursera_ICL_Certificate_Health Data Usage_V3XFWO53BYYT</x:v>
+        <x:v>Using Data for Healthcare Improvement</x:v>
       </x:c>
       <x:c r="E99" s="32" t="str">
         <x:v>J u l 2 4 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o U s i n g D a t a f o r H e a l t h c a r e I m p r o v e m e n t a n o n l i n e c o u r s e a u t h o r i z e d b y I m p e r i a l C o l l e g e L o n d o n a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d D r T h o m a s W o o d c o c k S e n i o r R e s e a r c h F e l l o w S c h o o l o f P u b l i c H e a l t h V e r i f y a t : h t t p s : / / c o u r s e r a . o r g / v e r i </x:v>
@@ -4445,11 +4517,17 @@
       <x:c r="I99" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J99" s="33"/>
-      <x:c r="K99" s="33"/>
-      <x:c r="L99" s="33"/>
+      <x:c r="J99" s="33" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="K99" s="33" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="L99" s="33" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="M99" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/V3XFWO53BYYT</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
@@ -4705,10 +4783,10 @@
         <x:v>Duke-Coursera_Telehealth_Cardiopulmonary Specialization DSEV3OLMXEMK.pdf</x:v>
       </x:c>
       <x:c r="C107" s="32" t="str">
-        <x:v>Duke</x:v>
+        <x:v>Duke University</x:v>
       </x:c>
       <x:c r="D107" s="32" t="str">
-        <x:v>Duke-Coursera_Telehealth_Cardiopulmonary Specialization DSEV3OLMXEMK</x:v>
+        <x:v>Telehealth: Essentials, Teamwork, and Cardiopulmonary Exam</x:v>
       </x:c>
       <x:c r="E107" s="32" t="str">
         <x:v>3 C o u r s e s T e l e h e a l t h C l i n i c a l E s s e n t i a l s T e l e h e a l t h : I n t e r p r o f e s s i o n a l T e a m - B a s e d C a r e T e l e h e a l t h : C a r d i o p u l m o n a r y A s s e s s m e n t D a n i e l O s t r o v s k y A s s o c i a t e P r o f e s s o r P e d i a t r i c s K a t h l e e n W a i t e P r o f e s s o r o f M e d i c i n e D i v i s i o n o f G e n e r a l I n t e r n a l M e d i c i n e A u g 3 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a </x:v>
@@ -4723,11 +4801,17 @@
       <x:c r="I107" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J107" s="33"/>
-      <x:c r="K107" s="33"/>
-      <x:c r="L107" s="33"/>
+      <x:c r="J107" s="33" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="K107" s="33" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="L107" s="33" t="n">
+        <x:v>12</x:v>
+      </x:c>
       <x:c r="M107" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/DSEV3OLMXEMK; estimativa derivada do tempo exibido: 1 meses com 3 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="108">
@@ -4738,10 +4822,10 @@
         <x:v>Duke-Coursera_Telehealth_Dermatology_Certificate_R2FTYV77JH0A.pdf</x:v>
       </x:c>
       <x:c r="C108" s="32" t="str">
-        <x:v>Duke</x:v>
+        <x:v>Duke University</x:v>
       </x:c>
       <x:c r="D108" s="32" t="str">
-        <x:v>Duke-Coursera_Telehealth_Dermatology_Certificate_R2FTYV77JH0A</x:v>
+        <x:v>Telehealth: Dermatology Assessment</x:v>
       </x:c>
       <x:c r="E108" s="32" t="str">
         <x:v>A u g 3 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o T e l e h e a l t h : D e r m a t o l o g y A s s e s s m e n t a n o n l i n e c o u r s e a u t h o r i z e d b y D u k e U n i v e r s i t y a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d D a n i e l O s t r o v s k y A s s o c i a t e P r o f e s s o r P e d i a t r i c s K a t h l e e n W a i t e P r o f e s s o r o f M e d i c i n e D i v i s i o n o f G e n e r a l I n t e r n a </x:v>
@@ -4756,11 +4840,17 @@
       <x:c r="I108" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J108" s="33"/>
-      <x:c r="K108" s="33"/>
-      <x:c r="L108" s="33"/>
+      <x:c r="J108" s="33" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K108" s="33" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L108" s="33" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="M108" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/R2FTYV77JH0A</x:v>
       </x:c>
     </x:row>
     <x:row r="109">
@@ -4771,10 +4861,10 @@
         <x:v>Duke-Coursera_Telehealth_Dermatology_Specialization Certificate_CG5I6U6HR05R..pdf</x:v>
       </x:c>
       <x:c r="C109" s="32" t="str">
-        <x:v>Duke</x:v>
+        <x:v>Duke University</x:v>
       </x:c>
       <x:c r="D109" s="32" t="str">
-        <x:v>Duke-Coursera_Telehealth_Dermatology_Specialization Certificate_CG5I6U6HR05R.</x:v>
+        <x:v>Telehealth: Essentials, Teamwork, and Dermatology</x:v>
       </x:c>
       <x:c r="E109" s="32" t="str">
         <x:v>3 C o u r s e s T e l e h e a l t h C l i n i c a l E s s e n t i a l s T e l e h e a l t h : I n t e r p r o f e s s i o n a l T e a m - B a s e d C a r e T e l e h e a l t h : D e r m a t o l o g y A s s e s s m e n t D a n i e l O s t r o v s k y A s s o c i a t e P r o f e s s o r P e d i a t r i c s K a t h l e e n W a i t e P r o f e s s o r o f M e d i c i n e D i v i s i o n o f G e n e r a l I n t e r n a l M e d i c i n e A u g 3 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o h a </x:v>
@@ -4790,15 +4880,17 @@
         <x:v>Extraído do documento</x:v>
       </x:c>
       <x:c r="J109" s="33" t="n">
-        <x:v>6</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="K109" s="33" t="n">
-        <x:v>6</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="L109" s="33" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="M109" s="32" t="str"/>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M109" s="32" t="str">
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/CG5I6U6HR05R; estimativa derivada do tempo exibido: 1 meses com 3 por semana para concluir</x:v>
+      </x:c>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="32" t="n">
@@ -4808,10 +4900,10 @@
         <x:v>Duke-Coursera_Telehealth_Musculoskeletal_Exam_Certificate_2J767H2OB448.pdf</x:v>
       </x:c>
       <x:c r="C110" s="32" t="str">
-        <x:v>Duke</x:v>
+        <x:v>Duke University</x:v>
       </x:c>
       <x:c r="D110" s="32" t="str">
-        <x:v>Duke-Coursera_Telehealth_Musculoskeletal_Exam_Certificate_2J767H2OB448</x:v>
+        <x:v>Telehealth: Musculoskeletal Assessment</x:v>
       </x:c>
       <x:c r="E110" s="32" t="str">
         <x:v>A u g 1 7 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o T e l e h e a l t h : M u s c u l o s k e l e t a l A s s e s s m e n t a n o n l i n e c o u r s e a u t h o r i z e d b y D u k e U n i v e r s i t y a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d D a n i e l O s t r o v s k y A s s o c i a t e P r o f e s s o r P e d i a t r i c s K a t h l e e n W a i t e P r o f e s s o r o f M e d i c i n e D i v i s i o n o f G e n e r a l I n </x:v>
@@ -4827,15 +4919,17 @@
         <x:v>Extraído do documento</x:v>
       </x:c>
       <x:c r="J110" s="33" t="n">
-        <x:v>7</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K110" s="33" t="n">
-        <x:v>7</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L110" s="33" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="M110" s="32" t="str"/>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="M110" s="32" t="str">
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/2J767H2OB448</x:v>
+      </x:c>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="32" t="n">
@@ -4845,10 +4939,10 @@
         <x:v>Duke-Coursera_Telehealth_Musculoskeletal_Specialization Certificate_ZVA616EKPRVQ.pdf</x:v>
       </x:c>
       <x:c r="C111" s="32" t="str">
-        <x:v>Duke</x:v>
+        <x:v>Duke University</x:v>
       </x:c>
       <x:c r="D111" s="32" t="str">
-        <x:v>Duke-Coursera_Telehealth_Musculoskeletal_Specialization Certificate_ZVA616EKPRVQ</x:v>
+        <x:v>Telehealth: Essentials, Teamwork, and Musculoskeletal Exam</x:v>
       </x:c>
       <x:c r="E111" s="32" t="str">
         <x:v>3 C o u r s e s T e l e h e a l t h C l i n i c a l E s s e n t i a l s T e l e h e a l t h : I n t e r p r o f e s s i o n a l T e a m - B a s e d C a r e T e l e h e a l t h : M u s c u l o s k e l e t a l A s s e s s m e n t D a n i e l O s t r o v s k y A s s o c i a t e P r o f e s s o r P e d i a t r i c s K a t h l e e n W a i t e P r o f e s s o r o f M e d i c i n e D i v i s i o n o f G e n e r a l I n t e r n a l M e d i c i n e A u g 1 7 , 2 0 2 6 P e d r o L a m o u n i e r S a m p </x:v>
@@ -4863,11 +4957,17 @@
       <x:c r="I111" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J111" s="33"/>
-      <x:c r="K111" s="33"/>
-      <x:c r="L111" s="33"/>
+      <x:c r="J111" s="33" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="K111" s="33" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="L111" s="33" t="n">
+        <x:v>12</x:v>
+      </x:c>
       <x:c r="M111" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/ZVA616EKPRVQ; estimativa derivada do tempo exibido: 1 meses com 3 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
@@ -4878,10 +4978,10 @@
         <x:v>Duke-Coursera_Telehealth_Neurological Exam Course_Certificate_UCSTLLOAX0QZ.pdf</x:v>
       </x:c>
       <x:c r="C112" s="32" t="str">
-        <x:v>Duke</x:v>
+        <x:v>Duke University</x:v>
       </x:c>
       <x:c r="D112" s="32" t="str">
-        <x:v>Duke-Coursera_Telehealth_Neurological Exam Course_Certificate_UCSTLLOAX0QZ</x:v>
+        <x:v>Telehealth: Neurological Exam Course</x:v>
       </x:c>
       <x:c r="E112" s="32" t="str">
         <x:v>A u g 1 7 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o T e l e h e a l t h : N e u r o l o g i c A s s e s s m e n t a n o n l i n e c o u r s e a u t h o r i z e d b y D u k e U n i v e r s i t y a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d D a n i e l O s t r o v s k y A s s o c i a t e P r o f e s s o r P e d i a t r i c s K a t h l e e n W a i t e P r o f e s s o r o f M e d i c i n e D i v i s i o n o f G e n e r a l I n t e r n a </x:v>
@@ -4900,7 +5000,7 @@
       <x:c r="K112" s="33"/>
       <x:c r="L112" s="33"/>
       <x:c r="M112" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/UCSTLLOAX0QZ</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
@@ -4911,10 +5011,10 @@
         <x:v>Duke-Coursera_Telehealth_Neurology_Certificate_UCSTLLOAX0QZ.pdf</x:v>
       </x:c>
       <x:c r="C113" s="32" t="str">
-        <x:v>Duke</x:v>
+        <x:v>Duke University</x:v>
       </x:c>
       <x:c r="D113" s="32" t="str">
-        <x:v>Duke-Coursera_Telehealth_Neurology_Certificate_UCSTLLOAX0QZ</x:v>
+        <x:v>Telehealth: Neurology</x:v>
       </x:c>
       <x:c r="E113" s="32" t="str">
         <x:v>3 C o u r s e s T e l e h e a l t h C l i n i c a l E s s e n t i a l s T e l e h e a l t h : I n t e r p r o f e s s i o n a l T e a m - B a s e d C a r e T e l e h e a l t h : N e u r o l o g i c A s s e s s m e n t D a n i e l O s t r o v s k y A s s o c i a t e P r o f e s s o r P e d i a t r i c s K a t h l e e n W a i t e P r o f e s s o r o f M e d i c i n e D i v i s i o n o f G e n e r a l I n t e r n a l M e d i c i n e A u g 1 7 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o h a </x:v>
@@ -4933,7 +5033,7 @@
       <x:c r="K113" s="33"/>
       <x:c r="L113" s="33"/>
       <x:c r="M113" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/UCSTLLOAX0QZ</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
@@ -6037,10 +6137,10 @@
         <x:v>HBS-Coursera_Effective Leadership_UQNUF9TGZVM9.pdf</x:v>
       </x:c>
       <x:c r="C147" s="32" t="str">
-        <x:v>HBS</x:v>
+        <x:v>Harvard Business School</x:v>
       </x:c>
       <x:c r="D147" s="32" t="str">
-        <x:v>HBS-Coursera_Effective Leadership_UQNUF9TGZVM9</x:v>
+        <x:v>Becoming an Effective Leader</x:v>
       </x:c>
       <x:c r="E147" s="32" t="str">
         <x:v>A u g 7 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o B e c o m i n g a n E f f e c t i v e L e a d e r a n o n l i n e c o u r s e a u t h o r i z e d b y H a r v a r d B u s i n e s s S c h o o l O n l i n e a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d H a r v a r d B u s i n e s s S c h o o l O n l i n e V e r i f y a t : h t t p s : / / c o u r s e r a . o r g / v e r i f y / U Q N U F 9 T G Z V M 9 C o u r s e r a h a s c o n f i r </x:v>
@@ -6055,11 +6155,17 @@
       <x:c r="I147" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J147" s="33"/>
-      <x:c r="K147" s="33"/>
-      <x:c r="L147" s="33"/>
+      <x:c r="J147" s="33" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K147" s="33" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L147" s="33" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="M147" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/UQNUF9TGZVM9</x:v>
       </x:c>
     </x:row>
     <x:row r="148">
@@ -6070,10 +6176,10 @@
         <x:v>HBS-Coursera_Intro to Leadership Specialization Certificate_53FFGZD92GQU.pdf</x:v>
       </x:c>
       <x:c r="C148" s="32" t="str">
-        <x:v>HBS</x:v>
+        <x:v>Harvard Business School</x:v>
       </x:c>
       <x:c r="D148" s="32" t="str">
-        <x:v>HBS-Coursera_Intro to Leadership Specialization Certificate_53FFGZD92GQU</x:v>
+        <x:v>Introduction to Leadership Principles</x:v>
       </x:c>
       <x:c r="E148" s="32" t="str">
         <x:v>2 C o u r s e s B e c o m i n g a n E ﬀ e c t i v e L e a d e r L e a d i n g H i g h - P e r f o r m i n g T e a m s H a r v a r d B u s i n e s s S c h o o l O n l i n e A u g 7 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o h a s s u c c e s s f u l l y c o m p l e t e d t h e o n l i n e S p e c i a l i z a t i o n I n t r o d u c t i o n t o L e a d e r s h i p P r i n c i p l e s T h i s s p e c i a l i z a t i o n , d e v e l o p e d b y H B S O n l i n e a n d o ﬀ e r e d t h r o u </x:v>
@@ -6088,11 +6194,17 @@
       <x:c r="I148" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J148" s="33"/>
-      <x:c r="K148" s="33"/>
-      <x:c r="L148" s="33"/>
+      <x:c r="J148" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="K148" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="L148" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
       <x:c r="M148" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/53FFGZD92GQU; estimativa derivada do tempo exibido: 1 meses com 10 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="149">
@@ -6483,10 +6595,10 @@
         <x:v>ICL-Coursera_Digital Health_Specialization Certificate CO5VFFKM5MQ6.pdf</x:v>
       </x:c>
       <x:c r="C161" s="32" t="str">
-        <x:v>ICL</x:v>
+        <x:v>Imperial College London</x:v>
       </x:c>
       <x:c r="D161" s="32" t="str">
-        <x:v>ICL-Coursera_Digital Health_Specialization Certificate CO5VFFKM5MQ6</x:v>
+        <x:v>Digital Health</x:v>
       </x:c>
       <x:c r="E161" s="32" t="str">
         <x:v>3 C o u r s e s I n t r o d u c t i o n t o D i g i t a l h e a l t h D e s i g n a n d I m p l e m e n t a t i o n o f D i g i t a l H e a l t h I n t e r v e n t i o n s E v a l u a t i o n o f D i g i t a l H e a l t h I n t e r v e n t i o n s A n a L u i s a N e v e s S e n i o r C l i n i c a l L e c t u r e r &amp; D i r e c t o r o f G l o b a l D i g i t a l H e a l t h U n i t S c h o o l o f P u b l i c H e a l t h A u g 7 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o h a s s u c c </x:v>
@@ -6501,11 +6613,17 @@
       <x:c r="I161" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J161" s="33"/>
-      <x:c r="K161" s="33"/>
-      <x:c r="L161" s="33"/>
+      <x:c r="J161" s="33" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="K161" s="33" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="L161" s="33" t="n">
+        <x:v>80</x:v>
+      </x:c>
       <x:c r="M161" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/CO5VFFKM5MQ6; estimativa derivada do tempo exibido: 2 meses com 10 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="162">
@@ -6549,10 +6667,10 @@
         <x:v>IllinoisMed-Coursera_Health Ecosystem 3O4Q2WIWVNSX.pdf</x:v>
       </x:c>
       <x:c r="C163" s="32" t="str">
-        <x:v>IllinoisMed</x:v>
+        <x:v>University of Illinois Chicago</x:v>
       </x:c>
       <x:c r="D163" s="32" t="str">
-        <x:v>IllinoisMed-Coursera_Health Ecosystem 3O4Q2WIWVNSX</x:v>
+        <x:v>Understanding the Healthcare Ecosystem</x:v>
       </x:c>
       <x:c r="E163" s="32" t="str">
         <x:v>J u l 2 6 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o U n d e r s t a n d i n g t h e H e a l t h c a r e E c o s y s t e m a n o n l i n e c o u r s e a u t h o r i z e d b y U n i v e r s i t y o f I l l i n o i s U r b a n a - C h a m p a i g n a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d S r i d h a r S e s h a d r i A l a n J . a n d J o y c e D . B a l t z E n d o w e d P r o f e s s o r a n d P r o f e s s o r o f B u s i n e s </x:v>
@@ -6567,11 +6685,17 @@
       <x:c r="I163" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J163" s="33"/>
-      <x:c r="K163" s="33"/>
-      <x:c r="L163" s="33"/>
+      <x:c r="J163" s="33" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="K163" s="33" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="L163" s="33" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="M163" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/3O4Q2WIWVNSX</x:v>
       </x:c>
     </x:row>
     <x:row r="164">
@@ -6871,10 +6995,10 @@
         <x:v>JHU-Coursera_Analysis of Programs_Certificate 3Z8RM8B5P6LS.pdf</x:v>
       </x:c>
       <x:c r="C173" s="32" t="str">
-        <x:v>JHU</x:v>
+        <x:v>Johns Hopkins University</x:v>
       </x:c>
       <x:c r="D173" s="32" t="str">
-        <x:v>JHU-Coursera_Analysis of Programs_Certificate 3Z8RM8B5P6LS</x:v>
+        <x:v>Analysis and Interpretation of Large-Scale Programs</x:v>
       </x:c>
       <x:c r="E173" s="32" t="str">
         <x:v>A u g 1 0 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o A n a l y s i s a n d I n t e r p r e t a t i o n o f L a r g e - S c a l e P r o g r a m s a n o n l i n e c o u r s e a u t h o r i z e d b y J o h n s H o p k i n s U n i v e r s i t y a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d A g b e s s i A m o u z o u - A s s o c i a t e P r o f e s s o r ; N e f f W a l k e r - S e n i o r S c i e n t i s t ; M e l i n d a M u n o s - A s </x:v>
@@ -6889,11 +7013,17 @@
       <x:c r="I173" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J173" s="33"/>
-      <x:c r="K173" s="33"/>
-      <x:c r="L173" s="33"/>
+      <x:c r="J173" s="33" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="K173" s="33" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="L173" s="33" t="n">
+        <x:v>21</x:v>
+      </x:c>
       <x:c r="M173" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/3Z8RM8B5P6LS</x:v>
       </x:c>
     </x:row>
     <x:row r="174">
@@ -6904,10 +7034,10 @@
         <x:v>JHU-Coursera_Biostatistics in PH_4XIVGLM9A4VF.pdf</x:v>
       </x:c>
       <x:c r="C174" s="32" t="str">
-        <x:v>JHU</x:v>
+        <x:v>Johns Hopkins University</x:v>
       </x:c>
       <x:c r="D174" s="32" t="str">
-        <x:v>JHU-Coursera_Biostatistics in PH_4XIVGLM9A4VF</x:v>
+        <x:v>Biostatistics in Public Health</x:v>
       </x:c>
       <x:c r="E174" s="32" t="str">
         <x:v>4 C o u r s e s S u m m a r y S t a t i s t i c s i n P u b l i c H e a l t h H y p o t h e s i s T e s t i n g i n P u b l i c H e a l t h S i m p l e R e g r e s s i o n A n a l y s i s i n P u b l i c H e a l t h M u l t i p l e R e g r e s s i o n A n a l y s i s i n P u b l i c H e a l t h J o h n M c G r e a d y , P h D , M S A s s o c i a t e S c i e n t i s t D e p a r t m e n t o f B i o s t a t i s t i c s A u g 8 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o h a s s u c c e s s </x:v>
@@ -6926,7 +7056,7 @@
       <x:c r="K174" s="33"/>
       <x:c r="L174" s="33"/>
       <x:c r="M174" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/4XIVGLM9A4VF</x:v>
       </x:c>
     </x:row>
     <x:row r="175">
@@ -6937,10 +7067,10 @@
         <x:v>JHU-Coursera_Evaluating Health Programs_Specializatin Certificate_9LMUYO3P4H4E.pdf</x:v>
       </x:c>
       <x:c r="C175" s="32" t="str">
-        <x:v>JHU</x:v>
+        <x:v>Johns Hopkins University</x:v>
       </x:c>
       <x:c r="D175" s="32" t="str">
-        <x:v>JHU-Coursera_Evaluating Health Programs_Specializatin Certificate_9LMUYO3P4H4E</x:v>
+        <x:v>Evaluating Large-Scale Health Programs</x:v>
       </x:c>
       <x:c r="E175" s="32" t="str">
         <x:v>6 C o u r s e s E v a l u a t i n g P u b l i c H e a l t h P r o g r a m s a t S c a l e P r o g r a m D e s i g n &amp; E v a l u a t i o n f o r H e a l t h S y s t e m s S t r e n g t h e n i n g A s s e s s i n g H e a l t h P r o g r a m D e l i v e r y H o u s e h o l d S u r v e y s f o r P r o g r a m E v a l u a t i o n i n L M I C s M e a s u r i n g a n d M o d e l i n g I m p a c t i n E v a l u a t i o n s A n a l y s i s a n d I n t e r p r e t a t i o n o f L a r g e - S c a l e P r </x:v>
@@ -6956,15 +7086,17 @@
         <x:v>Extraído do documento</x:v>
       </x:c>
       <x:c r="J175" s="33" t="n">
-        <x:v>4</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="K175" s="33" t="n">
-        <x:v>4</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="L175" s="33" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="M175" s="32" t="str"/>
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="M175" s="32" t="str">
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/9LMUYO3P4H4E; estimativa derivada do tempo exibido: 6 meses com 3 por semana para concluir</x:v>
+      </x:c>
     </x:row>
     <x:row r="176">
       <x:c r="A176" s="32" t="n">
@@ -6974,10 +7106,10 @@
         <x:v>JHU-Coursera_Health Program Delivery_Certificate 47FKHSCQYH5D.pdf</x:v>
       </x:c>
       <x:c r="C176" s="32" t="str">
-        <x:v>JHU</x:v>
+        <x:v>Johns Hopkins University</x:v>
       </x:c>
       <x:c r="D176" s="32" t="str">
-        <x:v>JHU-Coursera_Health Program Delivery_Certificate 47FKHSCQYH5D</x:v>
+        <x:v>Assessing Health Program Delivery</x:v>
       </x:c>
       <x:c r="E176" s="32" t="str">
         <x:v>A u g 1 0 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o A s s e s s i n g H e a l t h P r o g r a m D e l i v e r y a n o n l i n e c o u r s e a u t h o r i z e d b y J o h n s H o p k i n s U n i v e r s i t y a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d E l i z a b e t h H a z e l , A s s i s t a n t S c i e n t i s t , I n t e r n a t i o n a l H e a l t h | D i w a k a r M o h a n , A s s i s t a n t S c i e n t i s t , I n t e r n </x:v>
@@ -6992,11 +7124,17 @@
       <x:c r="I176" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J176" s="33"/>
-      <x:c r="K176" s="33"/>
-      <x:c r="L176" s="33"/>
+      <x:c r="J176" s="33" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="K176" s="33" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="L176" s="33" t="n">
+        <x:v>19</x:v>
+      </x:c>
       <x:c r="M176" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/47FKHSCQYH5D</x:v>
       </x:c>
     </x:row>
     <x:row r="177">
@@ -7007,10 +7145,10 @@
         <x:v>JHU-Coursera_PH Programs Evaluation_Certificate URX3MO9G7TX7.pdf</x:v>
       </x:c>
       <x:c r="C177" s="32" t="str">
-        <x:v>JHU</x:v>
+        <x:v>Johns Hopkins University</x:v>
       </x:c>
       <x:c r="D177" s="32" t="str">
-        <x:v>JHU-Coursera_PH Programs Evaluation_Certificate URX3MO9G7TX7</x:v>
+        <x:v>Evaluating Public Health Programs at Scale</x:v>
       </x:c>
       <x:c r="E177" s="32" t="str">
         <x:v>A u g 8 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o E v a l u a t i n g P u b l i c H e a l t h P r o g r a m s a t S c a l e a n o n l i n e c o u r s e a u t h o r i z e d b y J o h n s H o p k i n s U n i v e r s i t y a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d A g b e s s i A m o u z o u , P h D , M H S A s s o c i a t e P r o f e s s o r I n t e r n a t i o n a l H e a l t h N e f f W a l k e r , P h D S e n i o r S c i e n t i </x:v>
@@ -7025,11 +7163,17 @@
       <x:c r="I177" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J177" s="33"/>
-      <x:c r="K177" s="33"/>
-      <x:c r="L177" s="33"/>
+      <x:c r="J177" s="33" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="K177" s="33" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="L177" s="33" t="n">
+        <x:v>18</x:v>
+      </x:c>
       <x:c r="M177" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/URX3MO9G7TX7</x:v>
       </x:c>
     </x:row>
     <x:row r="178">
@@ -7040,10 +7184,10 @@
         <x:v>JHU-Coursera_Program Design and Evaluation_Certificate_N5X42IZWTN22.pdf</x:v>
       </x:c>
       <x:c r="C178" s="32" t="str">
-        <x:v>JHU</x:v>
+        <x:v>Johns Hopkins University</x:v>
       </x:c>
       <x:c r="D178" s="32" t="str">
-        <x:v>JHU-Coursera_Program Design and Evaluation_Certificate_N5X42IZWTN22</x:v>
+        <x:v>Program Design &amp; Evaluation for Health Systems Strengthening</x:v>
       </x:c>
       <x:c r="E178" s="32" t="str">
         <x:v>A u g 9 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o P r o g r a m D e s i g n &amp; E v a l u a t i o n f o r H e a l t h S y s t e m s S t r e n g t h e n i n g a n o n l i n e c o u r s e a u t h o r i z e d b y J o h n s H o p k i n s U n i v e r s i t y a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d T i m o t h y R o b e r t o n , D r P H , A s s i s t a n t S c i e n t i s t | J a y a G u p t a , P h D , H e a l t h S y s t e m s R e s </x:v>
@@ -7058,11 +7202,17 @@
       <x:c r="I178" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J178" s="33"/>
-      <x:c r="K178" s="33"/>
-      <x:c r="L178" s="33"/>
+      <x:c r="J178" s="33" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="K178" s="33" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="L178" s="33" t="n">
+        <x:v>7</x:v>
+      </x:c>
       <x:c r="M178" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/N5X42IZWTN22</x:v>
       </x:c>
     </x:row>
     <x:row r="179">
@@ -7417,10 +7567,10 @@
         <x:v>MichiganU-Coursera_Intro to Translational Science_Certificate_AI712ZU1D9CZ.pdf</x:v>
       </x:c>
       <x:c r="C189" s="32" t="str">
-        <x:v>MichiganU</x:v>
+        <x:v>University of Michigan</x:v>
       </x:c>
       <x:c r="D189" s="32" t="str">
-        <x:v>MichiganU-Coursera_Intro to Translational Science_Certificate_AI712ZU1D9CZ</x:v>
+        <x:v>Introduction to Translational Science</x:v>
       </x:c>
       <x:c r="E189" s="32" t="str">
         <x:v>A u g 4 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o I n t r o d u c t i o n t o T r a n s l a t i o n a l S c i e n c e a n o n l i n e c o u r s e a u t h o r i z e d b y U n i v e r s i t y o f M i c h i g a n a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d V i c k i E l l i n g r o d S e n i o r A s s o c i a t e D e a n C o l l e g e o f P h a r m a c y V e r i f y a t : h t t p s : / / c o u r s e r a . o r g / v e r i f y / A I 7 1 </x:v>
@@ -7435,11 +7585,17 @@
       <x:c r="I189" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J189" s="33"/>
-      <x:c r="K189" s="33"/>
-      <x:c r="L189" s="33"/>
+      <x:c r="J189" s="33" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="K189" s="33" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="L189" s="33" t="n">
+        <x:v>12</x:v>
+      </x:c>
       <x:c r="M189" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/AI712ZU1D9CZ</x:v>
       </x:c>
     </x:row>
     <x:row r="190">
@@ -8370,10 +8526,10 @@
         <x:v>Penn-Coursera_Healthcare Law Specialization Certificate VOUZB1AZBVL4.pdf</x:v>
       </x:c>
       <x:c r="C218" s="32" t="str">
-        <x:v>Penn</x:v>
+        <x:v>University of Pennsylvania</x:v>
       </x:c>
       <x:c r="D218" s="32" t="str">
-        <x:v>Penn-Coursera_Healthcare Law Specialization Certificate VOUZB1AZBVL4</x:v>
+        <x:v>Healthcare Law</x:v>
       </x:c>
       <x:c r="E218" s="32" t="str">
         <x:v>4 C o u r s e s U . S . H e a l t h L a w F u n d a m e n t a l s P r i v a c y L a w a n d H I P A A I n t e l l e c t u a l P r o p e r t y i n t h e H e a l t h c a r e I n d u s t r y C o m p a r a t i v e H e a l t h S y s t e m s T h e o d o r e R u g e r , J D D e a n a n d B e r n a r d G . S e g a l P r o f e s s o r o f L a w P e n n L a w L a u r e n S t e i n f e l d L e c t u r e r i n L a w R . P o l k W a g n e r P r o f e s s o r o f L a w A n g u s C o r b e t t A d j u n c t P </x:v>
@@ -8388,11 +8544,17 @@
       <x:c r="I218" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J218" s="33"/>
-      <x:c r="K218" s="33"/>
-      <x:c r="L218" s="33"/>
+      <x:c r="J218" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="K218" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="L218" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
       <x:c r="M218" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/VOUZB1AZBVL4; estimativa derivada do tempo exibido: 1 meses com 10 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="219">
@@ -8403,10 +8565,10 @@
         <x:v>Penn-Coursera_Intellectual Property in Healthcare_Certificate_ME8EBTCWCKTS.pdf</x:v>
       </x:c>
       <x:c r="C219" s="32" t="str">
-        <x:v>Penn</x:v>
+        <x:v>University of Pennsylvania</x:v>
       </x:c>
       <x:c r="D219" s="32" t="str">
-        <x:v>Penn-Coursera_Intellectual Property in Healthcare_Certificate_ME8EBTCWCKTS</x:v>
+        <x:v>Intellectual Property in the Healthcare Industry</x:v>
       </x:c>
       <x:c r="E219" s="32" t="str">
         <x:v>A u g 7 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o I n t e l l e c t u a l P r o p e r t y i n t h e H e a l t h c a r e I n d u s t r y a n o n l i n e n o n - c r e d i t c o u r s e a u t h o r i z e d b y U n i v e r s i t y o f P e n n s y l v a n i a a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d R . P o l k W a g n e r P r o f e s s o r o f L a w V e r i f y a t : h t t p s : / / c o u r s e r a . o r g / v e r i f y / M E 8 E B </x:v>
@@ -8421,11 +8583,17 @@
       <x:c r="I219" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J219" s="33"/>
-      <x:c r="K219" s="33"/>
-      <x:c r="L219" s="33"/>
+      <x:c r="J219" s="33" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="K219" s="33" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="L219" s="33" t="n">
+        <x:v>13</x:v>
+      </x:c>
       <x:c r="M219" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/ME8EBTCWCKTS</x:v>
       </x:c>
     </x:row>
     <x:row r="220">
@@ -9681,10 +9849,10 @@
         <x:v>Said-Oxford-Coursera_Agentic and GenAI_Certificate5YR8YBKNEOIC.pdf</x:v>
       </x:c>
       <x:c r="C257" s="32" t="str">
-        <x:v>Said</x:v>
+        <x:v>Saïd Business School, University of Oxford</x:v>
       </x:c>
       <x:c r="D257" s="32" t="str">
-        <x:v>Said-Oxford-Coursera_Agentic and GenAI_Certificate5YR8YBKNEOIC</x:v>
+        <x:v>Generative and Agentic AI</x:v>
       </x:c>
       <x:c r="E257" s="32" t="str">
         <x:v>A u g 1 4 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o G e n e r a t i v e a n d A g e n t i c A I a n o n l i n e c o u r s e a u t h o r i z e d b y S a ï d B u s i n e s s S c h o o l , U n i v e r s i t y o f O x f o r d a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d M a t t h i a s H o l w e g A m e r i c a n S t a n d a r d C o m p a n i e s P r o f e s s o r o f O p e r a t i o n s M a n a g e m e n t S a ï d B u s i n e s s S c h </x:v>
@@ -9699,11 +9867,17 @@
       <x:c r="I257" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J257" s="33"/>
-      <x:c r="K257" s="33"/>
-      <x:c r="L257" s="33"/>
+      <x:c r="J257" s="33" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="K257" s="33" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="L257" s="33" t="n">
+        <x:v>13</x:v>
+      </x:c>
       <x:c r="M257" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/5YR8YBKNEOIC</x:v>
       </x:c>
     </x:row>
     <x:row r="258">
@@ -9714,10 +9888,10 @@
         <x:v>Said-Oxford-Coursera_AI Essentials_Certificate EN2VCPK6A775.pdf</x:v>
       </x:c>
       <x:c r="C258" s="32" t="str">
-        <x:v>Said</x:v>
+        <x:v>Saïd Business School, University of Oxford</x:v>
       </x:c>
       <x:c r="D258" s="32" t="str">
-        <x:v>Said-Oxford-Coursera_AI Essentials_Certificate EN2VCPK6A775</x:v>
+        <x:v>AI Essentials</x:v>
       </x:c>
       <x:c r="E258" s="32" t="str">
         <x:v>A u g 1 3 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o A I E s s e n t i a l s a n o n l i n e c o u r s e a u t h o r i z e d b y S a ï d B u s i n e s s S c h o o l , U n i v e r s i t y o f O x f o r d a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d M a t t h i a s H o l w e g A m e r i c a n S t a n d a r d C o m p a n i e s P r o f e s s o r o f O p e r a t i o n s M a n a g e m e n t S a ï d B u s i n e s s S c h o o l U n i v e r s </x:v>
@@ -9732,11 +9906,17 @@
       <x:c r="I258" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J258" s="33"/>
-      <x:c r="K258" s="33"/>
-      <x:c r="L258" s="33"/>
+      <x:c r="J258" s="33" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="K258" s="33" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="L258" s="33" t="n">
+        <x:v>13</x:v>
+      </x:c>
       <x:c r="M258" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/EN2VCPK6A775</x:v>
       </x:c>
     </x:row>
     <x:row r="259">
@@ -9747,10 +9927,10 @@
         <x:v>Said-Oxford-Coursera_AI Governance_Certificate_FWGA4AWODSM4.pdf</x:v>
       </x:c>
       <x:c r="C259" s="32" t="str">
-        <x:v>Said</x:v>
+        <x:v>Saïd Business School, University of Oxford</x:v>
       </x:c>
       <x:c r="D259" s="32" t="str">
-        <x:v>Said-Oxford-Coursera_AI Governance_Certificate_FWGA4AWODSM4</x:v>
+        <x:v>AI Governance</x:v>
       </x:c>
       <x:c r="E259" s="32" t="str">
         <x:v>A u g 1 4 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o A I G o v e r n a n c e a n o n l i n e c o u r s e a u t h o r i z e d b y S a ï d B u s i n e s s S c h o o l , U n i v e r s i t y o f O x f o r d a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d M a t t h i a s H o l w e g A m e r i c a n S t a n d a r d C o m p a n i e s P r o f e s s o r o f O p e r a t i o n s M a n a g e m e n t S a ï d B u s i n e s s S c h o o l U n i v e r s </x:v>
@@ -9765,11 +9945,17 @@
       <x:c r="I259" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J259" s="33"/>
-      <x:c r="K259" s="33"/>
-      <x:c r="L259" s="33"/>
+      <x:c r="J259" s="33" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="K259" s="33" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="L259" s="33" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="M259" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/FWGA4AWODSM4</x:v>
       </x:c>
     </x:row>
     <x:row r="260">
@@ -9780,10 +9966,10 @@
         <x:v>Said-Oxford-Coursera_Specialization AI for Business_Certificate_FWGA4AWODSM4.pdf</x:v>
       </x:c>
       <x:c r="C260" s="32" t="str">
-        <x:v>Said</x:v>
+        <x:v>Saïd Business School, University of Oxford</x:v>
       </x:c>
       <x:c r="D260" s="32" t="str">
-        <x:v>Said-Oxford-Coursera_Specialization AI for Business_Certificate_FWGA4AWODSM4</x:v>
+        <x:v>AI for Business</x:v>
       </x:c>
       <x:c r="E260" s="32" t="str">
         <x:v>3 C o u r s e s A I E s s e n t i a l s G e n e r a t i v e a n d A g e n t i c A I A I G o v e r n a n c e M a t t h i a s H o l w e g A m e r i c a n S t a n d a r d C o m p a n i e s P r o f e s s o r o f O p e r a t i o n s M a n a g e m e n t S a ï d B u s i n e s s S c h o o l U n i v e r s i t y o f O x f o r d A u g 1 4 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o h a s s u c c e s s f u l l y c o m p l e t e d t h e o n l i n e S p e c i a l i z a t i o n A I F o u n d a t i o n </x:v>
@@ -9802,7 +9988,7 @@
       <x:c r="K260" s="33"/>
       <x:c r="L260" s="33"/>
       <x:c r="M260" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/FWGA4AWODSM4</x:v>
       </x:c>
     </x:row>
     <x:row r="261">
@@ -10397,10 +10583,10 @@
         <x:v>Stanford-Coursera RYUIMPUS3ZLR_Intro to Healthcare_Certificate.pdf</x:v>
       </x:c>
       <x:c r="C277" s="32" t="str">
-        <x:v>Stanford</x:v>
+        <x:v>Stanford Online / Stanford Medicine</x:v>
       </x:c>
       <x:c r="D277" s="32" t="str">
-        <x:v>Stanford-Coursera RYUIMPUS3ZLR_Intro to Healthcare_Certificate</x:v>
+        <x:v>Introduction to Healthcare</x:v>
       </x:c>
       <x:c r="E277" s="32" t="str">
         <x:v>J u l 2 8 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o I n t r o d u c t i o n t o H e a l t h c a r e a n o n l i n e c o u r s e a u t h o r i z e d b y S t a n f o r d U n i v e r s i t y a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d L a u r e n c e B a k e r , M i l d r e d C h o , N i g a m S h a h V e r i f y a t : h t t p s : / / c o u r s e r a . o r g / v e r i f y / R Y U I M P U S 3 Z L R C o u r s e r a h a s c o n f i r m e </x:v>
@@ -10415,11 +10601,17 @@
       <x:c r="I277" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J277" s="33"/>
-      <x:c r="K277" s="33"/>
-      <x:c r="L277" s="33"/>
+      <x:c r="J277" s="33" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="K277" s="33" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="L277" s="33" t="n">
+        <x:v>12</x:v>
+      </x:c>
       <x:c r="M277" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/RYUIMPUS3ZLR</x:v>
       </x:c>
     </x:row>
     <x:row r="278">
@@ -10430,10 +10622,10 @@
         <x:v>Stanford-Coursera_AI in Healthcare Capstone Certificate_9L3NBFUCKU4Q.pdf</x:v>
       </x:c>
       <x:c r="C278" s="32" t="str">
-        <x:v>Stanford</x:v>
+        <x:v>Stanford Online / Stanford Medicine</x:v>
       </x:c>
       <x:c r="D278" s="32" t="str">
-        <x:v>Stanford-Coursera_AI in Healthcare Capstone Certificate_9L3NBFUCKU4Q</x:v>
+        <x:v>AI in Healthcare Capstone</x:v>
       </x:c>
       <x:c r="E278" s="32" t="str">
         <x:v>A u g 2 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o A I i n H e a l t h c a r e C a p s t o n e a n o n l i n e c o u r s e a u t h o r i z e d b y S t a n f o r d U n i v e r s i t y a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d L a u r e n c e B a k e r , M a t t h e w L u n g r e n , N i g a m S h a h , S e r e n a Y e u n g a n d T i n a H e r n a n d e z - B o u s s a r d V e r i f y a t : h t t p s : / / c o u r s e r a . o r g / </x:v>
@@ -10448,11 +10640,17 @@
       <x:c r="I278" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J278" s="33"/>
-      <x:c r="K278" s="33"/>
-      <x:c r="L278" s="33"/>
+      <x:c r="J278" s="33" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="K278" s="33" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="L278" s="33" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="M278" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/9L3NBFUCKU4Q</x:v>
       </x:c>
     </x:row>
     <x:row r="279">
@@ -10463,10 +10661,10 @@
         <x:v>Stanford-Coursera_AI in Healthcare Specialization Certificate_7GM7A9EIJ9W4.pdf</x:v>
       </x:c>
       <x:c r="C279" s="32" t="str">
-        <x:v>Stanford</x:v>
+        <x:v>Stanford Online / Stanford Medicine</x:v>
       </x:c>
       <x:c r="D279" s="32" t="str">
-        <x:v>Stanford-Coursera_AI in Healthcare Specialization Certificate_7GM7A9EIJ9W4</x:v>
+        <x:v>AI in Healthcare</x:v>
       </x:c>
       <x:c r="E279" s="32" t="str">
         <x:v>5 C o u r s e s I n t r o d u c t i o n t o H e a l t h c a r e I n t r o d u c t i o n t o C l i n i c a l D a t a F u n d a m e n t a l s o f M a c h i n e L e a r n i n g f o r H e a l t h c a r e E v a l u a t i o n s o f A I A p p l i c a t i o n s i n H e a l t h c a r e A I i n H e a l t h c a r e C a p s t o n e N i g a m H . S h a h , M B B S , P h D A s s o c i a t e P r o f e s s o r o f M e d i c i n e ( B i o m e d i c a l I n f o r m a t i c s ) A u g 2 , 2 0 2 6 P e d r o L a m o </x:v>
@@ -10481,11 +10679,17 @@
       <x:c r="I279" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J279" s="33"/>
-      <x:c r="K279" s="33"/>
-      <x:c r="L279" s="33"/>
+      <x:c r="J279" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="K279" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="L279" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
       <x:c r="M279" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/7GM7A9EIJ9W4; estimativa derivada do tempo exibido: 1 meses com 10 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="280">
@@ -10496,10 +10700,10 @@
         <x:v>Stanford-Coursera_Certificate_Fundamentals of ML in HC_MYZ6GPXEFO5H.pdf</x:v>
       </x:c>
       <x:c r="C280" s="32" t="str">
-        <x:v>Stanford</x:v>
+        <x:v>Stanford Online / Stanford Medicine</x:v>
       </x:c>
       <x:c r="D280" s="32" t="str">
-        <x:v>Stanford-Coursera_Certificate_Fundamentals of ML in HC_MYZ6GPXEFO5H</x:v>
+        <x:v>Fundamentals of Machine Learning for Healthcare</x:v>
       </x:c>
       <x:c r="E280" s="32" t="str">
         <x:v>A u g 1 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o F u n d a m e n t a l s o f M a c h i n e L e a r n i n g f o r H e a l t h c a r e a n o n l i n e c o u r s e a u t h o r i z e d b y S t a n f o r d U n i v e r s i t y a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d M a t t h e w L u n g r e n A s s o c i a t e P r o f e s s o r D e p a r t m e n t o f R a d i o l o g y S e r e n a Y e u n g A s s i s t a n t P r o f e s s o r B i o </x:v>
@@ -10515,15 +10719,17 @@
         <x:v>Extraído do documento</x:v>
       </x:c>
       <x:c r="J280" s="33" t="n">
-        <x:v>5</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="K280" s="33" t="n">
-        <x:v>5</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="L280" s="33" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="M280" s="32" t="str"/>
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="M280" s="32" t="str">
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/MYZ6GPXEFO5H</x:v>
+      </x:c>
     </x:row>
     <x:row r="281">
       <x:c r="A281" s="32" t="n">
@@ -10533,10 +10739,10 @@
         <x:v>Stanford-Coursera_Evaluations of AI in HC_Certificate_DW8FFD7QA2IZ.pdf</x:v>
       </x:c>
       <x:c r="C281" s="32" t="str">
-        <x:v>Stanford</x:v>
+        <x:v>Stanford Online / Stanford Medicine</x:v>
       </x:c>
       <x:c r="D281" s="32" t="str">
-        <x:v>Stanford-Coursera_Evaluations of AI in HC_Certificate_DW8FFD7QA2IZ</x:v>
+        <x:v>Evaluations of AI Applications in Healthcare</x:v>
       </x:c>
       <x:c r="E281" s="32" t="str">
         <x:v>A u g 1 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o E v a l u a t i o n s o f A I A p p l i c a t i o n s i n H e a l t h c a r e a n o n l i n e c o u r s e a u t h o r i z e d b y S t a n f o r d U n i v e r s i t y a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d T i n a H e r n a n d e z - B o u s s a r d A s s o c i a t e P r o f e s s o r M e d i c i n e ( B i o m e d i c a l I n f o r m a t i c s ) , o f B i o m e d i c a l D a t a </x:v>
@@ -10551,11 +10757,17 @@
       <x:c r="I281" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J281" s="33"/>
-      <x:c r="K281" s="33"/>
-      <x:c r="L281" s="33"/>
+      <x:c r="J281" s="33" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="K281" s="33" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="L281" s="33" t="n">
+        <x:v>11</x:v>
+      </x:c>
       <x:c r="M281" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/DW8FFD7QA2IZ</x:v>
       </x:c>
     </x:row>
     <x:row r="282">
@@ -10636,10 +10848,10 @@
         <x:v>Stanford-Coursera_PCA Specialization Certificate E8700K9GB2WD.pdf</x:v>
       </x:c>
       <x:c r="C284" s="32" t="str">
-        <x:v>Stanford</x:v>
+        <x:v>Stanford Online / Stanford Medicine</x:v>
       </x:c>
       <x:c r="D284" s="32" t="str">
-        <x:v>Stanford-Coursera_PCA Specialization Certificate E8700K9GB2WD</x:v>
+        <x:v>Palliative Care Always</x:v>
       </x:c>
       <x:c r="E284" s="32" t="str">
         <x:v>5 C o u r s e s E s s e n t i a l s o f P a l l i a t i v e C a r e S y m p t o m M a n a g e m e n t i n P a l l i a t i v e C a r e T r a n s i t i o n s i n C a r e f r o m S u r v i v o r s h i p t o H o s p i c e S u p p o r t i n g F a m i l i e s a n d C a r e g i v e r s P a l l i a t i v e C a r e A l w a y s C a p s t o n e C o u r s e K a v i t h a R a m c h a n d r a n M D , C l i n i c a l A s s o c i a t e P r o f e s s o r , S t a n f o r d M e d i c i n e A u g 3 0 , 2 0 2 6 P e </x:v>
@@ -10654,11 +10866,17 @@
       <x:c r="I284" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J284" s="33"/>
-      <x:c r="K284" s="33"/>
-      <x:c r="L284" s="33"/>
+      <x:c r="J284" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="K284" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="L284" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
       <x:c r="M284" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/E8700K9GB2WD; estimativa derivada do tempo exibido: 1 meses com 10 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="285">
@@ -10669,10 +10887,10 @@
         <x:v>Stanford-Coursera_Supporting Caregiver Health_Certificate_O8W0ZHG0J5II.pdf</x:v>
       </x:c>
       <x:c r="C285" s="32" t="str">
-        <x:v>Stanford</x:v>
+        <x:v>Stanford Online / Stanford Medicine</x:v>
       </x:c>
       <x:c r="D285" s="32" t="str">
-        <x:v>Stanford-Coursera_Supporting Caregiver Health_Certificate_O8W0ZHG0J5II</x:v>
+        <x:v>Supporting Families and Caregivers</x:v>
       </x:c>
       <x:c r="E285" s="32" t="str">
         <x:v>A u g 3 0 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o S u p p o r t i n g F a m i l i e s a n d C a r e g i v e r s a n o n l i n e c o u r s e a u t h o r i z e d b y S t a n f o r d O n l i n e a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d K a v i t h a R a m c h a n d r a n C l i n i c a l A s s o c i a t e P r o f e s s o r O n c o l o g y J a n D e N o f r i o P h D P r o g r a m M a n a g e r P a l l i a t i v e C a r e A l w a y </x:v>
@@ -10687,11 +10905,17 @@
       <x:c r="I285" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J285" s="33"/>
-      <x:c r="K285" s="33"/>
-      <x:c r="L285" s="33"/>
+      <x:c r="J285" s="33" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="K285" s="33" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="L285" s="33" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="M285" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/O8W0ZHG0J5II</x:v>
       </x:c>
     </x:row>
     <x:row r="286">
@@ -10702,10 +10926,10 @@
         <x:v>Stanford-Coursera_Symptom Management_CertificateLYD5V9AWXRXS.pdf</x:v>
       </x:c>
       <x:c r="C286" s="32" t="str">
-        <x:v>Stanford</x:v>
+        <x:v>Stanford Online / Stanford Medicine</x:v>
       </x:c>
       <x:c r="D286" s="32" t="str">
-        <x:v>Stanford-Coursera_Symptom Management_CertificateLYD5V9AWXRXS</x:v>
+        <x:v>Symptom Management in Palliative Care</x:v>
       </x:c>
       <x:c r="E286" s="32" t="str">
         <x:v>A u g 2 9 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o S y m p t o m M a n a g e m e n t i n P a l l i a t i v e C a r e a n o n l i n e c o u r s e a u t h o r i z e d b y S t a n f o r d O n l i n e a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d J a n D e N o f r i o , J o s h u a F r o n k , K a v i t h a R a m c h a n d r a n , M a n u e l a K o g o n V e r i f y a t : h t t p s : / / c o u r s e r a . o r g / v e r i f y / L Y D 5 V </x:v>
@@ -10720,11 +10944,17 @@
       <x:c r="I286" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J286" s="33"/>
-      <x:c r="K286" s="33"/>
-      <x:c r="L286" s="33"/>
+      <x:c r="J286" s="33" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="K286" s="33" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="L286" s="33" t="n">
+        <x:v>9</x:v>
+      </x:c>
       <x:c r="M286" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/LYD5V9AWXRXS</x:v>
       </x:c>
     </x:row>
     <x:row r="287">
@@ -10805,10 +11035,10 @@
         <x:v>Stanfrod-Coursera_Supporting families and caregivers Certificate_O8W0ZHG0J5II.pdf</x:v>
       </x:c>
       <x:c r="C289" s="32" t="str">
-        <x:v>Stanfrod</x:v>
+        <x:v>Stanford Online / Stanford Medicine</x:v>
       </x:c>
       <x:c r="D289" s="32" t="str">
-        <x:v>Stanfrod-Coursera_Supporting families and caregivers Certificate_O8W0ZHG0J5II</x:v>
+        <x:v>Supporting Families and Caregivers</x:v>
       </x:c>
       <x:c r="E289" s="32" t="str">
         <x:v>A u g 3 0 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o S u p p o r t i n g F a m i l i e s a n d C a r e g i v e r s a n o n l i n e c o u r s e a u t h o r i z e d b y S t a n f o r d O n l i n e a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d K a v i t h a R a m c h a n d r a n C l i n i c a l A s s o c i a t e P r o f e s s o r O n c o l o g y J a n D e N o f r i o P h D P r o g r a m M a n a g e r P a l l i a t i v e C a r e A l w a y </x:v>
@@ -10823,11 +11053,17 @@
       <x:c r="I289" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J289" s="33"/>
-      <x:c r="K289" s="33"/>
-      <x:c r="L289" s="33"/>
+      <x:c r="J289" s="33" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="K289" s="33" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="L289" s="33" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="M289" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/O8W0ZHG0J5II</x:v>
       </x:c>
     </x:row>
     <x:row r="290">
@@ -11234,10 +11470,10 @@
         <x:v>U-M-Coursera_Translating Research to communities Certificate_WWZOYLD9AB26.pdf</x:v>
       </x:c>
       <x:c r="C302" s="32" t="str">
-        <x:v>U</x:v>
+        <x:v>University of Michigan</x:v>
       </x:c>
       <x:c r="D302" s="32" t="str">
-        <x:v>U-M-Coursera_Translating Research to communities Certificate_WWZOYLD9AB26</x:v>
+        <x:v>Translating Research to Communities</x:v>
       </x:c>
       <x:c r="E302" s="32" t="str">
         <x:v>A u g 2 9 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o T r a n s l a t i n g R e s e a r c h t o C o m m u n i t i e s a n o n l i n e c o u r s e a u t h o r i z e d b y U n i v e r s i t y o f M i c h i g a n a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d V i c k i E l l i n g r o d J o h n G i d e o n S e a r l e P r o f e s s o r o f P h a r m a c y , D e a n ; P r o f e s s o r o f P s y c h i a t r y C o l l e g e o f P h a r m a c </x:v>
@@ -11252,11 +11488,17 @@
       <x:c r="I302" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J302" s="33"/>
-      <x:c r="K302" s="33"/>
-      <x:c r="L302" s="33"/>
+      <x:c r="J302" s="33" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K302" s="33" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="L302" s="33" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="M302" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/WWZOYLD9AB26</x:v>
       </x:c>
     </x:row>
     <x:row r="303">
@@ -11267,10 +11509,10 @@
         <x:v>U-M-Coursera_Translating Research to Patients Certificate_IKDNWXUCALFA.pdf</x:v>
       </x:c>
       <x:c r="C303" s="32" t="str">
-        <x:v>U</x:v>
+        <x:v>University of Michigan</x:v>
       </x:c>
       <x:c r="D303" s="32" t="str">
-        <x:v>U-M-Coursera_Translating Research to Patients Certificate_IKDNWXUCALFA</x:v>
+        <x:v>Translating Research to Patients</x:v>
       </x:c>
       <x:c r="E303" s="32" t="str">
         <x:v>A u g 2 9 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o T r a n s l a t i n g R e s e a r c h t o P a t i e n t s a n o n l i n e c o u r s e a u t h o r i z e d b y U n i v e r s i t y o f M i c h i g a n a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d V i c k i E l l i n g r o d J o h n G i d e o n S e a r l e P r o f e s s o r o f P h a r m a c y , D e a n ; P r o f e s s o r o f P s y c h i a t r y C o l l e g e o f P h a r m a c y , M </x:v>
@@ -11285,11 +11527,17 @@
       <x:c r="I303" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J303" s="33"/>
-      <x:c r="K303" s="33"/>
-      <x:c r="L303" s="33"/>
+      <x:c r="J303" s="33" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K303" s="33" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="L303" s="33" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="M303" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/IKDNWXUCALFA</x:v>
       </x:c>
     </x:row>
     <x:row r="304">
@@ -11300,10 +11548,10 @@
         <x:v>U-M-Coursera_Translating Research to Policy Certificate_0HXUUQIWD1P7.pdf</x:v>
       </x:c>
       <x:c r="C304" s="32" t="str">
-        <x:v>U</x:v>
+        <x:v>University of Michigan</x:v>
       </x:c>
       <x:c r="D304" s="32" t="str">
-        <x:v>U-M-Coursera_Translating Research to Policy Certificate_0HXUUQIWD1P7</x:v>
+        <x:v>Translating Research to Healthcare Policy</x:v>
       </x:c>
       <x:c r="E304" s="32" t="str">
         <x:v>A u g 2 9 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o T r a n s l a t i n g R e s e a r c h t o H e a l t h c a r e P o l i c y a n o n l i n e c o u r s e a u t h o r i z e d b y U n i v e r s i t y o f M i c h i g a n a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d V i c k i E l l i n g r o d J o h n G i d e o n S e a r l e P r o f e s s o r o f P h a r m a c y , D e a n ; P r o f e s s o r o f P s y c h i a t r y C o l l e g e o f P h </x:v>
@@ -11319,15 +11567,17 @@
         <x:v>Extraído do documento</x:v>
       </x:c>
       <x:c r="J304" s="33" t="n">
-        <x:v>0</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="K304" s="33" t="n">
-        <x:v>0</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="L304" s="33" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M304" s="32" t="str"/>
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="M304" s="32" t="str">
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/0HXUUQIWD1P7</x:v>
+      </x:c>
     </x:row>
     <x:row r="305">
       <x:c r="A305" s="32" t="n">
@@ -11337,10 +11587,10 @@
         <x:v>U-M-Coursera_Translational Research for humans_Certificate 7MIVPFC1VTQR.pdf</x:v>
       </x:c>
       <x:c r="C305" s="32" t="str">
-        <x:v>U</x:v>
+        <x:v>University of Michigan</x:v>
       </x:c>
       <x:c r="D305" s="32" t="str">
-        <x:v>U-M-Coursera_Translational Research for humans_Certificate 7MIVPFC1VTQR</x:v>
+        <x:v>Translating Basic Research into Research for Humans</x:v>
       </x:c>
       <x:c r="E305" s="32" t="str">
         <x:v>A u g 1 3 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o T r a n s l a t i n g B a s i c R e s e a r c h i n t o R e s e a r c h f o r H u m a n s a n o n l i n e c o u r s e a u t h o r i z e d b y U n i v e r s i t y o f M i c h i g a n a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d V i c k i E l l i n g r o d S e n i o r A s s o c i a t e D e a n C o l l e g e o f P h a r m a c y V e r i f y a t : h t t p s : / / c o u r s e r a . o r g </x:v>
@@ -11355,11 +11605,17 @@
       <x:c r="I305" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J305" s="33"/>
-      <x:c r="K305" s="33"/>
-      <x:c r="L305" s="33"/>
+      <x:c r="J305" s="33" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="K305" s="33" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L305" s="33" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="M305" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/7MIVPFC1VTQR</x:v>
       </x:c>
     </x:row>
     <x:row r="306">
@@ -11370,10 +11626,10 @@
         <x:v>U-M-Coursera_Translational Science Specialization Certificate_IXQRUXCLXP3K.pdf</x:v>
       </x:c>
       <x:c r="C306" s="32" t="str">
-        <x:v>U</x:v>
+        <x:v>University of Michigan</x:v>
       </x:c>
       <x:c r="D306" s="32" t="str">
-        <x:v>U-M-Coursera_Translational Science Specialization Certificate_IXQRUXCLXP3K</x:v>
+        <x:v>Translational Science</x:v>
       </x:c>
       <x:c r="E306" s="32" t="str">
         <x:v>5 C o u r s e s I n t r o d u c t i o n t o T r a n s l a t i o n a l S c i e n c e T r a n s l a t i n g B a s i c R e s e a r c h i n t o R e s e a r c h f o r H u m a n s T r a n s l a t i n g R e s e a r c h t o P a t i e n t s T r a n s l a t i n g R e s e a r c h t o C o m m u n i t i e s T r a n s l a t i n g R e s e a r c h t o H e a l t h c a r e P o l i c y V i c k i E l l i n g r o d S e n i o r A s s o c i a t e D e a n C o l l e g e o f P h a r m a c y A u g 2 9 , 2 0 2 6 P e d r o </x:v>
@@ -11388,11 +11644,17 @@
       <x:c r="I306" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J306" s="33"/>
-      <x:c r="K306" s="33"/>
-      <x:c r="L306" s="33"/>
+      <x:c r="J306" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="K306" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="L306" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
       <x:c r="M306" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/IXQRUXCLXP3K; estimativa derivada do tempo exibido: 1 meses com 10 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="307">
@@ -12020,10 +12282,10 @@
         <x:v>Yale-Coursera_Global Health Essentials_Certificate_YJ26WLVD3O3K.pdf</x:v>
       </x:c>
       <x:c r="C326" s="32" t="str">
-        <x:v>Yale</x:v>
+        <x:v>Yale University</x:v>
       </x:c>
       <x:c r="D326" s="32" t="str">
-        <x:v>Yale-Coursera_Global Health Essentials_Certificate_YJ26WLVD3O3K</x:v>
+        <x:v>Essentials of Global Health</x:v>
       </x:c>
       <x:c r="E326" s="32" t="str">
         <x:v>A u g 5 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o E s s e n t i a l s o f G l o b a l H e a l t h a n o n l i n e c o u r s e a u t h o r i z e d b y Y a l e U n i v e r s i t y a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d R i c h a r d S k o l n i k F o r m e r L e c t u r e r , D e p a r t m e n t o f H e a l t h P o l i c y a n d M a n a g e m e n t , Y a l e S c h o o l o f P u b l i c H e a l t h a n d L e c t u r e r i n t h e </x:v>
@@ -12038,11 +12300,17 @@
       <x:c r="I326" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="J326" s="33"/>
-      <x:c r="K326" s="33"/>
-      <x:c r="L326" s="33"/>
+      <x:c r="J326" s="33" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="K326" s="33" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="L326" s="33" t="n">
+        <x:v>39</x:v>
+      </x:c>
       <x:c r="M326" s="32" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/YJ26WLVD3O3K</x:v>
       </x:c>
     </x:row>
     <x:row r="327">
@@ -12084,7 +12352,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04c05768bace4641"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5633b7ec466c4e6b"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Completar dados dos certificados Coursera
</commit_message>
<xml_diff>
--- a/ACG_UNIFENAS_Medicina.xlsx
+++ b/ACG_UNIFENAS_Medicina.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R21a864e93ff341f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regras UNIFENAS" sheetId="2" r:id="R47d6610fc2e44920"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Certificados" sheetId="3" r:id="R91ad27624040493b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluídos" sheetId="4" r:id="R4acaf79ad5f24e18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pendências" sheetId="5" r:id="R31012f932d1f4daa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R0a96d4fe3c794ad9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regras UNIFENAS" sheetId="2" r:id="R88288ccc0e96487b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Certificados" sheetId="3" r:id="Rf93a249f3de3485d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluídos" sheetId="4" r:id="R439b4e79e4304ccd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pendências" sheetId="5" r:id="Rf6674072e94e46b0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -467,7 +467,7 @@
       </x:c>
       <x:c r="B6" s="16" t="n">
         <x:f>SUM('Certificados'!$K$2:$K$389)</x:f>
-        <x:v>2110.5</x:v>
+        <x:v>2244.5</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -476,7 +476,7 @@
       </x:c>
       <x:c r="B7" s="16" t="n">
         <x:f>SUM('Certificados'!$M$2:$M$389)</x:f>
-        <x:v>2110.5</x:v>
+        <x:v>2244.5</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -485,7 +485,7 @@
       </x:c>
       <x:c r="B8" s="16" t="n">
         <x:f>B3-B7</x:f>
-        <x:v>-1660.5</x:v>
+        <x:v>-1794.5</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -520,11 +520,11 @@
       </x:c>
       <x:c r="C12" s="30" t="n">
         <x:f>SUMIF('Certificados'!$H$2:$H$389,A12,'Certificados'!$K$2:$K$389)</x:f>
-        <x:v>1360.25</x:v>
+        <x:v>1494.25</x:v>
       </x:c>
       <x:c r="D12" s="30" t="n">
         <x:f>SUMIF('Certificados'!$H$2:$H$389,A12,'Certificados'!$M$2:$M$389)</x:f>
-        <x:v>1360.25</x:v>
+        <x:v>1494.25</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2118,7 +2118,7 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="N26" s="32" t="str">
-        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/K99N55L2EZNG; estimativa derivada do tempo exibido: 1 meses com 10 por semana para concluir</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/K99N55L2EZNG; duração exibida: 1 meses com 10 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -3501,7 +3501,9 @@
       <x:c r="E64" s="32" t="str">
         <x:v>Revenue Cycle, Billing, and Coding</x:v>
       </x:c>
-      <x:c r="F64" s="32" t="str"/>
+      <x:c r="F64" s="32" t="str">
+        <x:v>Patient registration; revenue cycle management; medical coding; billing; claims processing; and denial management.</x:v>
+      </x:c>
       <x:c r="G64" s="32" t="str"/>
       <x:c r="H64" s="32" t="str">
         <x:v>Grupo 1 — Ensino</x:v>
@@ -3542,7 +3544,7 @@
         <x:v>Revenue Cycle, Billing, and Coding</x:v>
       </x:c>
       <x:c r="F65" s="32" t="str">
-        <x:v>J u n 2 8 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o R e v e n u e C y c l e , B i l l i n g , a n d C o d i n g u m c u r s o o n - l i n e a u t o r i z a d o p e l a J o h n s H o p k i n s U n i v e r s i t y e m i n i s t r a d o a t r a v é s d a C o u r s e r a c o n c l u i u c o m s u c e s s o o P r o g r a m a d e c u r s o s i n t e g r a d o s M a u r a M c G u i r e , M D , C P C , F A C P E x e c u t i v e D i r e c t o r O J H P S t r a t e g i c L e a r n i n g C e n t </x:v>
+        <x:v>Patient registration; revenue cycle management; medical coding; billing; claims processing; and denial management.</x:v>
       </x:c>
       <x:c r="G65" s="32" t="str"/>
       <x:c r="H65" s="32" t="str">
@@ -3606,7 +3608,7 @@
         <x:v>72</x:v>
       </x:c>
       <x:c r="N66" s="32" t="str">
-        <x:v>Coursera: https://www.coursera.org/account/accomplishments/professional-cert/P7PRAOBUU4L9; estimativa derivada do tempo exibido: 6 meses com 3 por semana para concluir</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/professional-cert/P7PRAOBUU4L9; duração exibida: 6 meses com 3 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -3648,7 +3650,7 @@
         <x:v>72</x:v>
       </x:c>
       <x:c r="N67" s="32" t="str">
-        <x:v>Coursera: https://www.coursera.org/account/accomplishments/professional-cert/P7PRAOBUU4L9; estimativa derivada do tempo exibido: 6 meses com 3 por semana para concluir</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/professional-cert/P7PRAOBUU4L9; duração exibida: 6 meses com 3 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -4616,7 +4618,7 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="N94" s="32" t="str">
-        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/8BH1XC5QBHPD; estimativa derivada do tempo exibido: 1 meses com 10 por semana para concluir</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/8BH1XC5QBHPD; duração exibida: 1 meses com 10 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
@@ -4634,7 +4636,7 @@
         <x:v>Leading Healthcare Quality and Safety</x:v>
       </x:c>
       <x:c r="F95" s="32" t="str">
-        <x:v>J u l 2 1 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o L e a d i n g H e a l t h c a r e Q u a l i t y a n d S a f e t y a n o n l i n e c o u r s e a u t h o r i z e d b y T h e G e o r g e W a s h i n g t o n U n i v e r s i t y a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d G r e g o r y P a w l s o n C l i n i c a l P r o f e s s o r o f M e d i c i n e a n d E x e c u t i v e C o a c h G W S c h o o l o f N u r s i n g J e a n J o h </x:v>
+        <x:v>Patient safety; health informatics; healthcare administration; measurement systems; change management; and organizational change.</x:v>
       </x:c>
       <x:c r="G95" s="32" t="str"/>
       <x:c r="H95" s="32" t="str">
@@ -4718,7 +4720,7 @@
         <x:v>Quality Improvement in Healthcare</x:v>
       </x:c>
       <x:c r="F97" s="32" t="str">
-        <x:v>3 C o u r s e s I n t r o d u c t i o n t o Q u a l i t y I m p r o v e m e n t i n H e a l t h c a r e U s i n g D a t a f o r H e a l t h c a r e I m p r o v e m e n t Q u a l i t y I m p r o v e m e n t f o r P o p u l a t i o n H e a l t h D r T h o m a s W o o d c o c k S e n i o r R e s e a r c h F e l l o w S c h o o l o f P u b l i c H e a l t h J u l 2 4 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o h a s s u c c e s s f u l l y c o m p l e t e d t h e o n l i n e S p e c i a l i </x:v>
+        <x:v>Introduction to quality improvement in healthcare; using data for healthcare improvement; and quality improvement for population health.</x:v>
       </x:c>
       <x:c r="G97" s="32" t="str"/>
       <x:c r="H97" s="32" t="str">
@@ -4740,7 +4742,7 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="N97" s="32" t="str">
-        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/2RUAK3DPGYVQ; estimativa derivada do tempo exibido: 1 meses com 10 por semana para concluir</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/2RUAK3DPGYVQ; duração exibida: 1 meses com 10 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
@@ -4760,7 +4762,7 @@
         <x:v>Introduction to Quality Improvement in Healthcare</x:v>
       </x:c>
       <x:c r="F98" s="32" t="str">
-        <x:v>J u l 2 2 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o I n t r o d u c t i o n t o Q u a l i t y I m p r o v e m e n t i n H e a l t h c a r e a n o n l i n e c o u r s e a u t h o r i z e d b y I m p e r i a l C o l l e g e L o n d o n a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d D r T h o m a s W o o d c o c k S e n i o r R e s e a r c h F e l l o w S c h o o l o f P u b l i c H e a l t h V e r i f y a t : h t t p s : / / c o u r s e </x:v>
+        <x:v>Fundamentals of quality improvement in healthcare and methods for initiating improvement projects.</x:v>
       </x:c>
       <x:c r="G98" s="32" t="str"/>
       <x:c r="H98" s="32" t="str">
@@ -4802,7 +4804,7 @@
         <x:v>Using Data for Healthcare Improvement</x:v>
       </x:c>
       <x:c r="F99" s="32" t="str">
-        <x:v>J u l 2 4 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o U s i n g D a t a f o r H e a l t h c a r e I m p r o v e m e n t a n o n l i n e c o u r s e a u t h o r i z e d b y I m p e r i a l C o l l e g e L o n d o n a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d D r T h o m a s W o o d c o c k S e n i o r R e s e a r c h F e l l o w S c h o o l o f P u b l i c H e a l t h V e r i f y a t : h t t p s : / / c o u r s e r a . o r g / v e r i </x:v>
+        <x:v>Using healthcare data to identify problems, measure performance, and guide improvement.</x:v>
       </x:c>
       <x:c r="G99" s="32" t="str"/>
       <x:c r="H99" s="32" t="str">
@@ -5132,7 +5134,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="N107" s="32" t="str">
-        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/DSEV3OLMXEMK; estimativa derivada do tempo exibido: 1 meses com 3 por semana para concluir</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/DSEV3OLMXEMK; duração exibida: 1 meses com 3 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="108">
@@ -5216,7 +5218,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="N109" s="32" t="str">
-        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/CG5I6U6HR05R; estimativa derivada do tempo exibido: 1 meses com 3 por semana para concluir</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/CG5I6U6HR05R; duração exibida: 1 meses com 3 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="110">
@@ -5300,7 +5302,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="N111" s="32" t="str">
-        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/ZVA616EKPRVQ; estimativa derivada do tempo exibido: 1 meses com 3 por semana para concluir</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/ZVA616EKPRVQ; duração exibida: 1 meses com 3 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
@@ -5317,10 +5319,10 @@
         <x:v>Duke University</x:v>
       </x:c>
       <x:c r="E112" s="32" t="str">
-        <x:v>Telehealth: Neurological Exam Course</x:v>
+        <x:v>Telehealth: Neurologic Assessment</x:v>
       </x:c>
       <x:c r="F112" s="32" t="str">
-        <x:v>A u g 1 7 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o T e l e h e a l t h : N e u r o l o g i c A s s e s s m e n t a n o n l i n e c o u r s e a u t h o r i z e d b y D u k e U n i v e r s i t y a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d D a n i e l O s t r o v s k y A s s o c i a t e P r o f e s s o r P e d i a t r i c s K a t h l e e n W a i t e P r o f e s s o r o f M e d i c i n e D i v i s i o n o f G e n e r a l I n t e r n a </x:v>
+        <x:v>Perform a virtual neurological assessment; discuss the advantages and limitations of a virtual neurological assessment; describe the benefits of telehealth visits for patients with neurological concerns or conditions.</x:v>
       </x:c>
       <x:c r="G112" s="32" t="str"/>
       <x:c r="H112" s="32" t="str">
@@ -5332,11 +5334,17 @@
       <x:c r="J112" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="K112" s="33"/>
-      <x:c r="L112" s="33"/>
-      <x:c r="M112" s="33"/>
+      <x:c r="K112" s="33" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L112" s="33" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="M112" s="33" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="N112" s="32" t="str">
-        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/UCSTLLOAX0QZ</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/UCSTLLOAX0QZ; página do curso: https://www.coursera.org/learn/telehealth-neurologic-assessment; duração exibida: 2 horas para completar</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
@@ -5353,10 +5361,10 @@
         <x:v>Duke University</x:v>
       </x:c>
       <x:c r="E113" s="32" t="str">
-        <x:v>Telehealth: Neurology</x:v>
+        <x:v>Telehealth: Essentials, Teamwork, and Neurologic Exam</x:v>
       </x:c>
       <x:c r="F113" s="32" t="str">
-        <x:v>3 C o u r s e s T e l e h e a l t h C l i n i c a l E s s e n t i a l s T e l e h e a l t h : I n t e r p r o f e s s i o n a l T e a m - B a s e d C a r e T e l e h e a l t h : N e u r o l o g i c A s s e s s m e n t D a n i e l O s t r o v s k y A s s o c i a t e P r o f e s s o r P e d i a t r i c s K a t h l e e n W a i t e P r o f e s s o r o f M e d i c i n e D i v i s i o n o f G e n e r a l I n t e r n a l M e d i c i n e A u g 1 7 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o h a </x:v>
+        <x:v>Prepare and conduct telehealth video visits; describe team-based telehealth care; perform physical neurologic exams remotely; identify the benefits and limitations of telehealth visits.</x:v>
       </x:c>
       <x:c r="G113" s="32" t="str"/>
       <x:c r="H113" s="32" t="str">
@@ -5368,11 +5376,17 @@
       <x:c r="J113" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="K113" s="33"/>
-      <x:c r="L113" s="33"/>
-      <x:c r="M113" s="33"/>
+      <x:c r="K113" s="33" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="L113" s="33" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M113" s="33" t="n">
+        <x:v>12</x:v>
+      </x:c>
       <x:c r="N113" s="32" t="str">
-        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/UCSTLLOAX0QZ</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/UCSTLLOAX0QZ; página do curso: https://www.coursera.org/specializations/telehealth-neurologic-essentials-teamwork; duração exibida: 4 semanas com 3 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
@@ -6648,7 +6662,7 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="N148" s="32" t="str">
-        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/53FFGZD92GQU; estimativa derivada do tempo exibido: 1 meses com 10 por semana para concluir</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/53FFGZD92GQU; duração exibida: 1 meses com 10 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="149">
@@ -7084,7 +7098,7 @@
         <x:v>Digital Health</x:v>
       </x:c>
       <x:c r="F161" s="32" t="str">
-        <x:v>3 C o u r s e s I n t r o d u c t i o n t o D i g i t a l h e a l t h D e s i g n a n d I m p l e m e n t a t i o n o f D i g i t a l H e a l t h I n t e r v e n t i o n s E v a l u a t i o n o f D i g i t a l H e a l t h I n t e r v e n t i o n s A n a L u i s a N e v e s S e n i o r C l i n i c a l L e c t u r e r &amp; D i r e c t o r o f G l o b a l D i g i t a l H e a l t h U n i t S c h o o l o f P u b l i c H e a l t h A u g 7 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o h a s s u c c </x:v>
+        <x:v>Introduction to digital health; design and implementation of digital health interventions; and evaluation of digital health interventions.</x:v>
       </x:c>
       <x:c r="G161" s="32" t="str"/>
       <x:c r="H161" s="32" t="str">
@@ -7106,7 +7120,7 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="N161" s="32" t="str">
-        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/CO5VFFKM5MQ6; estimativa derivada do tempo exibido: 2 meses com 10 por semana para concluir</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/CO5VFFKM5MQ6; duração exibida: 2 meses com 10 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="162">
@@ -7520,7 +7534,7 @@
         <x:v>Analysis and Interpretation of Large-Scale Programs</x:v>
       </x:c>
       <x:c r="F173" s="32" t="str">
-        <x:v>A u g 1 0 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o A n a l y s i s a n d I n t e r p r e t a t i o n o f L a r g e - S c a l e P r o g r a m s a n o n l i n e c o u r s e a u t h o r i z e d b y J o h n s H o p k i n s U n i v e r s i t y a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d A g b e s s i A m o u z o u - A s s o c i a t e P r o f e s s o r ; N e f f W a l k e r - S e n i o r S c i e n t i s t ; M e l i n d a M u n o s - A s </x:v>
+        <x:v>Analysis and interpretation of large-scale health programs and their data.</x:v>
       </x:c>
       <x:c r="G173" s="32" t="str"/>
       <x:c r="H173" s="32" t="str">
@@ -7562,7 +7576,7 @@
         <x:v>Biostatistics in Public Health</x:v>
       </x:c>
       <x:c r="F174" s="32" t="str">
-        <x:v>4 C o u r s e s S u m m a r y S t a t i s t i c s i n P u b l i c H e a l t h H y p o t h e s i s T e s t i n g i n P u b l i c H e a l t h S i m p l e R e g r e s s i o n A n a l y s i s i n P u b l i c H e a l t h M u l t i p l e R e g r e s s i o n A n a l y s i s i n P u b l i c H e a l t h J o h n M c G r e a d y , P h D , M S A s s o c i a t e S c i e n t i s t D e p a r t m e n t o f B i o s t a t i s t i c s A u g 8 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o h a s s u c c e s s </x:v>
+        <x:v>Calculate summary statistics for biomedical and public health data; interpret written and visual presentations of statistical data; evaluate and interpret regression methods; choose the appropriate statistical method for a research question.</x:v>
       </x:c>
       <x:c r="G174" s="32" t="str"/>
       <x:c r="H174" s="32" t="str">
@@ -7574,11 +7588,17 @@
       <x:c r="J174" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="K174" s="33"/>
-      <x:c r="L174" s="33"/>
-      <x:c r="M174" s="33"/>
+      <x:c r="K174" s="33" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="L174" s="33" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="M174" s="33" t="n">
+        <x:v>80</x:v>
+      </x:c>
       <x:c r="N174" s="32" t="str">
-        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/4XIVGLM9A4VF</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/4XIVGLM9A4VF; página do curso: https://www.coursera.org/specializations/biostatistics-public-health; duração exibida: 2 meses com 10 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="175">
@@ -7620,7 +7640,7 @@
         <x:v>72</x:v>
       </x:c>
       <x:c r="N175" s="32" t="str">
-        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/9LMUYO3P4H4E; estimativa derivada do tempo exibido: 6 meses com 3 por semana para concluir</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/9LMUYO3P4H4E; duração exibida: 6 meses com 3 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="176">
@@ -7640,7 +7660,7 @@
         <x:v>Assessing Health Program Delivery</x:v>
       </x:c>
       <x:c r="F176" s="32" t="str">
-        <x:v>A u g 1 0 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o A s s e s s i n g H e a l t h P r o g r a m D e l i v e r y a n o n l i n e c o u r s e a u t h o r i z e d b y J o h n s H o p k i n s U n i v e r s i t y a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d E l i z a b e t h H a z e l , A s s i s t a n t S c i e n t i s t , I n t e r n a t i o n a l H e a l t h | D i w a k a r M o h a n , A s s i s t a n t S c i e n t i s t , I n t e r n </x:v>
+        <x:v>Assessment of health program delivery, including implementation and program performance.</x:v>
       </x:c>
       <x:c r="G176" s="32" t="str"/>
       <x:c r="H176" s="32" t="str">
@@ -7682,7 +7702,7 @@
         <x:v>Evaluating Public Health Programs at Scale</x:v>
       </x:c>
       <x:c r="F177" s="32" t="str">
-        <x:v>A u g 8 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o E v a l u a t i n g P u b l i c H e a l t h P r o g r a m s a t S c a l e a n o n l i n e c o u r s e a u t h o r i z e d b y J o h n s H o p k i n s U n i v e r s i t y a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d A g b e s s i A m o u z o u , P h D , M H S A s s o c i a t e P r o f e s s o r I n t e r n a t i o n a l H e a l t h N e f f W a l k e r , P h D S e n i o r S c i e n t i </x:v>
+        <x:v>Evaluation of public health programs at scale, using indicators, methods, and evidence to assess results.</x:v>
       </x:c>
       <x:c r="G177" s="32" t="str"/>
       <x:c r="H177" s="32" t="str">
@@ -7724,7 +7744,7 @@
         <x:v>Program Design &amp; Evaluation for Health Systems Strengthening</x:v>
       </x:c>
       <x:c r="F178" s="32" t="str">
-        <x:v>A u g 9 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o P r o g r a m D e s i g n &amp; E v a l u a t i o n f o r H e a l t h S y s t e m s S t r e n g t h e n i n g a n o n l i n e c o u r s e a u t h o r i z e d b y J o h n s H o p k i n s U n i v e r s i t y a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d T i m o t h y R o b e r t o n , D r P H , A s s i s t a n t S c i e n t i s t | J a y a G u p t a , P h D , H e a l t h S y s t e m s R e s </x:v>
+        <x:v>Program design and evaluation for health systems strengthening; planning, measurement, and interpretation of program results.</x:v>
       </x:c>
       <x:c r="G178" s="32" t="str"/>
       <x:c r="H178" s="32" t="str">
@@ -9172,7 +9192,7 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="N217" s="32" t="str">
-        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/VOUZB1AZBVL4; estimativa derivada do tempo exibido: 1 meses com 10 por semana para concluir</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/VOUZB1AZBVL4; duração exibida: 1 meses com 10 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="218">
@@ -10677,10 +10697,10 @@
         <x:v>Saïd Business School, University of Oxford</x:v>
       </x:c>
       <x:c r="E258" s="32" t="str">
-        <x:v>AI for Business</x:v>
+        <x:v>AI Foundations for Business Professionals</x:v>
       </x:c>
       <x:c r="F258" s="32" t="str">
-        <x:v>3 C o u r s e s A I E s s e n t i a l s G e n e r a t i v e a n d A g e n t i c A I A I G o v e r n a n c e M a t t h i a s H o l w e g A m e r i c a n S t a n d a r d C o m p a n i e s P r o f e s s o r o f O p e r a t i o n s M a n a g e m e n t S a ï d B u s i n e s s S c h o o l U n i v e r s i t y o f O x f o r d A u g 1 4 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o h a s s u c c e s s f u l l y c o m p l e t e d t h e o n l i n e S p e c i a l i z a t i o n A I F o u n d a t i o n </x:v>
+        <x:v>Understand core concepts of AI, machine learning, and deep learning and their strategic business value; distinguish generative and agentic AI from traditional models; apply ethical considerations and governance strategies; assess and manage AI risks, including system failures and bias.</x:v>
       </x:c>
       <x:c r="G258" s="32" t="str"/>
       <x:c r="H258" s="32" t="str">
@@ -10692,11 +10712,17 @@
       <x:c r="J258" s="32" t="str">
         <x:v>Extraído do documento</x:v>
       </x:c>
-      <x:c r="K258" s="33"/>
-      <x:c r="L258" s="33"/>
-      <x:c r="M258" s="33"/>
+      <x:c r="K258" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="L258" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="M258" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
       <x:c r="N258" s="32" t="str">
-        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/FWGA4AWODSM4</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/FWGA4AWODSM4; página do curso: https://www.coursera.org/specializations/ai-foundations-business-professionals; duração exibida: 4 semanas com 10 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="259">
@@ -11390,7 +11416,7 @@
         <x:v>AI in Healthcare Capstone</x:v>
       </x:c>
       <x:c r="F276" s="32" t="str">
-        <x:v>A u g 2 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o A I i n H e a l t h c a r e C a p s t o n e a n o n l i n e c o u r s e a u t h o r i z e d b y S t a n f o r d U n i v e r s i t y a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d L a u r e n c e B a k e r , M a t t h e w L u n g r e n , N i g a m S h a h , S e r e n a Y e u n g a n d T i n a H e r n a n d e z - B o u s s a r d V e r i f y a t : h t t p s : / / c o u r s e r a . o r g / </x:v>
+        <x:v>Applied capstone integrating artificial intelligence concepts for healthcare problem-solving and evaluation.</x:v>
       </x:c>
       <x:c r="G276" s="32" t="str"/>
       <x:c r="H276" s="32" t="str">
@@ -11454,7 +11480,7 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="N277" s="32" t="str">
-        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/7GM7A9EIJ9W4; estimativa derivada do tempo exibido: 1 meses com 10 por semana para concluir</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/7GM7A9EIJ9W4; duração exibida: 1 meses com 10 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="278">
@@ -11496,7 +11522,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="N278" s="32" t="str">
-        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/FZV2SBU6I8NI; estimativa derivada do tempo exibido: 5 horas (aproximadamente)</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/FZV2SBU6I8NI; duração exibida: 5 horas (aproximadamente)</x:v>
       </x:c>
     </x:row>
     <x:row r="279">
@@ -11622,7 +11648,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="N281" s="32" t="str">
-        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/WFZW6W7MXCAN; estimativa derivada do tempo exibido: 11 horas (aproximadamente)</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/WFZW6W7MXCAN; duração exibida: 11 horas (aproximadamente)</x:v>
       </x:c>
     </x:row>
     <x:row r="282">
@@ -11706,7 +11732,7 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="N283" s="32" t="str">
-        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/E8700K9GB2WD; estimativa derivada do tempo exibido: 1 meses com 10 por semana para concluir</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/E8700K9GB2WD; duração exibida: 1 meses com 10 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="284">
@@ -11832,7 +11858,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="N286" s="32" t="str">
-        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/OYTO0JAKNOFA; estimativa derivada do tempo exibido: 10 horas (aproximadamente)</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/verify/OYTO0JAKNOFA; duração exibida: 10 horas (aproximadamente)</x:v>
       </x:c>
     </x:row>
     <x:row r="287">
@@ -12556,7 +12582,7 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="N305" s="32" t="str">
-        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/IXQRUXCLXP3K; estimativa derivada do tempo exibido: 1 meses com 10 por semana para concluir</x:v>
+        <x:v>Coursera: https://www.coursera.org/account/accomplishments/specialization/IXQRUXCLXP3K; duração exibida: 1 meses com 10 por semana para concluir</x:v>
       </x:c>
     </x:row>
     <x:row r="306">
@@ -13250,7 +13276,7 @@
         <x:v>Essentials of Global Health</x:v>
       </x:c>
       <x:c r="F325" s="32" t="str">
-        <x:v>A u g 5 , 2 0 2 6 P e d r o L a m o u n i e r S a m p a i o E s s e n t i a l s o f G l o b a l H e a l t h a n o n l i n e c o u r s e a u t h o r i z e d b y Y a l e U n i v e r s i t y a n d o f f e r e d t h r o u g h C o u r s e r a h a s s u c c e s s f u l l y c o m p l e t e d R i c h a r d S k o l n i k F o r m e r L e c t u r e r , D e p a r t m e n t o f H e a l t h P o l i c y a n d M a n a g e m e n t , Y a l e S c h o o l o f P u b l i c H e a l t h a n d L e c t u r e r i n t h e </x:v>
+        <x:v>Global health determinants, health systems, disease burden, and strategies to improve population health.</x:v>
       </x:c>
       <x:c r="G325" s="32" t="str"/>
       <x:c r="H325" s="32" t="str">
@@ -13317,7 +13343,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb129e16c7bb24d8c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R103faf6a78d1499c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15456,7 +15482,7 @@
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="24" t="str">
-        <x:v>Duke-Coursera_Telehealth_Neurological Exam Course_Certificate_UCSTLLOAX0QZ.pdf</x:v>
+        <x:v>DUNS Resolved Inquiry # 10536566 (Case # 10601194) - Update for LAMOUNI.pdf</x:v>
       </x:c>
       <x:c r="B78" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -15471,7 +15497,7 @@
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="24" t="str">
-        <x:v>Duke-Coursera_Telehealth_Neurology_Certificate_UCSTLLOAX0QZ.pdf</x:v>
+        <x:v>E-mail confirmation sent by Alpha.pdf</x:v>
       </x:c>
       <x:c r="B79" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -15486,7 +15512,7 @@
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="24" t="str">
-        <x:v>DUNS Resolved Inquiry # 10536566 (Case # 10601194) - Update for LAMOUNI.pdf</x:v>
+        <x:v>E-mail from Alison.pdf</x:v>
       </x:c>
       <x:c r="B80" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -15501,10 +15527,10 @@
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="24" t="str">
-        <x:v>E-mail confirmation sent by Alpha.pdf</x:v>
+        <x:v>e1acc2cd-ba6a-4a63-8230-37366add71b1_eb96ae20cd844243b17a7d4ffb8e6c57_LLPC_Badge.png</x:v>
       </x:c>
       <x:c r="B81" s="24" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>PDF/imagem sem texto extraível</x:v>
       </x:c>
       <x:c r="C81" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -15516,7 +15542,7 @@
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="24" t="str">
-        <x:v>E-mail from Alison.pdf</x:v>
+        <x:v>EADV_00042657_certificate.pdf</x:v>
       </x:c>
       <x:c r="B82" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -15531,10 +15557,10 @@
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="24" t="str">
-        <x:v>e1acc2cd-ba6a-4a63-8230-37366add71b1_eb96ae20cd844243b17a7d4ffb8e6c57_LLPC_Badge.png</x:v>
+        <x:v>EGS003_Pedro Lamounier Sampaio_Participant_WPP__20260704-204242.pdf</x:v>
       </x:c>
       <x:c r="B83" s="24" t="str">
-        <x:v>PDF/imagem sem texto extraível</x:v>
+        <x:v>Carga horária não localizada</x:v>
       </x:c>
       <x:c r="C83" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -15546,7 +15572,7 @@
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="24" t="str">
-        <x:v>EADV_00042657_certificate.pdf</x:v>
+        <x:v>Ementa Curso Auditoria SES.pdf</x:v>
       </x:c>
       <x:c r="B84" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -15561,7 +15587,7 @@
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="24" t="str">
-        <x:v>EGS003_Pedro Lamounier Sampaio_Participant_WPP__20260704-204242.pdf</x:v>
+        <x:v>Ementa Curso POP-T-SVS-012.pdf</x:v>
       </x:c>
       <x:c r="B85" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -15576,7 +15602,7 @@
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="24" t="str">
-        <x:v>Ementa Curso Auditoria SES.pdf</x:v>
+        <x:v>Ementa Inspeção SVSS.pdf</x:v>
       </x:c>
       <x:c r="B86" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -15591,7 +15617,7 @@
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="24" t="str">
-        <x:v>Ementa Curso POP-T-SVS-012.pdf</x:v>
+        <x:v>EPICourses_OSHAin Healthcare and BPT_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B87" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -15606,7 +15632,7 @@
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="24" t="str">
-        <x:v>Ementa Inspeção SVSS.pdf</x:v>
+        <x:v>fd91e062-545f-0a1b-40b2-14937c01b355_file.pdf</x:v>
       </x:c>
       <x:c r="B88" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -15621,7 +15647,7 @@
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="24" t="str">
-        <x:v>EPICourses_OSHAin Healthcare and BPT_Certificate.pdf</x:v>
+        <x:v>FDCE-UFMG_Certificado_Extensão_Tributação Previdenciária_2020.10.pdf</x:v>
       </x:c>
       <x:c r="B89" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -15636,7 +15662,7 @@
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="24" t="str">
-        <x:v>fd91e062-545f-0a1b-40b2-14937c01b355_file.pdf</x:v>
+        <x:v>form-q-svs-005-v-00-programa-de-auditoria-interna.pdf</x:v>
       </x:c>
       <x:c r="B90" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -15651,7 +15677,7 @@
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="24" t="str">
-        <x:v>FDCE-UFMG_Certificado_Extensão_Tributação Previdenciária_2020.10.pdf</x:v>
+        <x:v>form-q-svs-006-v-00-relatorio-de-auditoria-interna.pdf</x:v>
       </x:c>
       <x:c r="B91" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -15666,10 +15692,10 @@
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="24" t="str">
-        <x:v>form-q-svs-005-v-00-programa-de-auditoria-interna.pdf</x:v>
+        <x:v>GHLC_HC WF Productivity and Quality_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B92" s="24" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>PDF/imagem sem texto extraível</x:v>
       </x:c>
       <x:c r="C92" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -15681,10 +15707,10 @@
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="24" t="str">
-        <x:v>form-q-svs-006-v-00-relatorio-de-auditoria-interna.pdf</x:v>
+        <x:v>GHTC_Infrastructure and Good Governance_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B93" s="24" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>PDF/imagem sem texto extraível</x:v>
       </x:c>
       <x:c r="C93" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -15696,10 +15722,10 @@
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="24" t="str">
-        <x:v>GHLC_HC WF Productivity and Quality_Certificate.pdf</x:v>
+        <x:v>GIACC_ Common types of corruption in project construction Certificate.pdf</x:v>
       </x:c>
       <x:c r="B94" s="24" t="str">
-        <x:v>PDF/imagem sem texto extraível</x:v>
+        <x:v>Carga horária não localizada</x:v>
       </x:c>
       <x:c r="C94" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -15711,10 +15737,10 @@
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="24" t="str">
-        <x:v>GHTC_Infrastructure and Good Governance_Certificate.pdf</x:v>
+        <x:v>GIACC_Benefits and Requirements of ISO 37301_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B95" s="24" t="str">
-        <x:v>PDF/imagem sem texto extraível</x:v>
+        <x:v>Carga horária não localizada</x:v>
       </x:c>
       <x:c r="C95" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -15726,7 +15752,7 @@
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="24" t="str">
-        <x:v>GIACC_ Common types of corruption in project construction Certificate.pdf</x:v>
+        <x:v>GIACC_Construction and Procurement Contracts_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B96" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -15741,7 +15767,7 @@
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="24" t="str">
-        <x:v>GIACC_Benefits and Requirements of ISO 37301_Certificate.pdf</x:v>
+        <x:v>GIACC_Construction Corruption Prevention Certificate.pdf</x:v>
       </x:c>
       <x:c r="B97" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -15756,7 +15782,7 @@
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="24" t="str">
-        <x:v>GIACC_Construction and Procurement Contracts_Certificate.pdf</x:v>
+        <x:v>GIACC_Corruption in Procurement Certificate.pdf</x:v>
       </x:c>
       <x:c r="B98" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -15771,7 +15797,7 @@
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="24" t="str">
-        <x:v>GIACC_Construction Corruption Prevention Certificate.pdf</x:v>
+        <x:v>GIACC_Corruption Investigation in Procurement_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B99" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -15786,7 +15812,7 @@
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="24" t="str">
-        <x:v>GIACC_Corruption in Procurement Certificate.pdf</x:v>
+        <x:v>GIACC_Mod11_Corruption Dilemmas_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B100" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -15801,7 +15827,7 @@
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="24" t="str">
-        <x:v>GIACC_Corruption Investigation in Procurement_Certificate.pdf</x:v>
+        <x:v>GIACC_Module 3_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B101" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -15816,7 +15842,7 @@
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="24" t="str">
-        <x:v>GIACC_Mod11_Corruption Dilemmas_Certificate.pdf</x:v>
+        <x:v>GICR-1 Certificate of Completion - WHO Academy.pdf</x:v>
       </x:c>
       <x:c r="B102" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -15831,7 +15857,7 @@
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="24" t="str">
-        <x:v>GIACC_Module 3_Certificate.pdf</x:v>
+        <x:v>GICR-O Certificate of Completion - WHO Academy.pdf</x:v>
       </x:c>
       <x:c r="B103" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -15846,10 +15872,10 @@
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="24" t="str">
-        <x:v>GICR-1 Certificate of Completion - WHO Academy.pdf</x:v>
+        <x:v>Global Health Governance Certificate.pdf</x:v>
       </x:c>
       <x:c r="B104" s="24" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>PDF/imagem sem texto extraível</x:v>
       </x:c>
       <x:c r="C104" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -15861,7 +15887,7 @@
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="24" t="str">
-        <x:v>GICR-O Certificate of Completion - WHO Academy.pdf</x:v>
+        <x:v>Global Infrastructure Anti-Corruption Centre Module 2 Certificate.pdf</x:v>
       </x:c>
       <x:c r="B105" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -15876,10 +15902,10 @@
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="24" t="str">
-        <x:v>Global Health Governance Certificate.pdf</x:v>
+        <x:v>Global Infrastructure Anti-Corruption Centre.pdf</x:v>
       </x:c>
       <x:c r="B106" s="24" t="str">
-        <x:v>PDF/imagem sem texto extraível</x:v>
+        <x:v>Carga horária não localizada</x:v>
       </x:c>
       <x:c r="C106" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -15891,10 +15917,10 @@
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="24" t="str">
-        <x:v>Global Infrastructure Anti-Corruption Centre Module 2 Certificate.pdf</x:v>
+        <x:v>Glossary_Modern_Project_Management_Microsoft365.zip</x:v>
       </x:c>
       <x:c r="B107" s="24" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>PDF/imagem sem texto extraível</x:v>
       </x:c>
       <x:c r="C107" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -15906,7 +15932,7 @@
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="24" t="str">
-        <x:v>Global Infrastructure Anti-Corruption Centre.pdf</x:v>
+        <x:v>HIPAA_Training_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B108" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -15921,10 +15947,10 @@
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="24" t="str">
-        <x:v>Glossary_Modern_Project_Management_Microsoft365.zip</x:v>
+        <x:v>HomeTown Health Certificate.pdf</x:v>
       </x:c>
       <x:c r="B109" s="24" t="str">
-        <x:v>PDF/imagem sem texto extraível</x:v>
+        <x:v>Carga horária não localizada</x:v>
       </x:c>
       <x:c r="C109" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -15936,7 +15962,7 @@
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="24" t="str">
-        <x:v>HIPAA_Training_Certificate.pdf</x:v>
+        <x:v>HomeTown Health_Care Coordination and Continuity.pdf</x:v>
       </x:c>
       <x:c r="B110" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -15951,10 +15977,10 @@
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="24" t="str">
-        <x:v>HomeTown Health Certificate.pdf</x:v>
+        <x:v>HSC_Curso sobre avaliação biológica ISO 10993_certificado-3533631.pdf</x:v>
       </x:c>
       <x:c r="B111" s="24" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>PDF/imagem sem texto extraível</x:v>
       </x:c>
       <x:c r="C111" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -15966,10 +15992,10 @@
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="24" t="str">
-        <x:v>HomeTown Health_Care Coordination and Continuity.pdf</x:v>
+        <x:v>HSC_Curso sobre Avaliação Clínica ISO 10993_certificado-3533419.pdf</x:v>
       </x:c>
       <x:c r="B112" s="24" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>PDF/imagem sem texto extraível</x:v>
       </x:c>
       <x:c r="C112" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -15981,7 +16007,7 @@
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="24" t="str">
-        <x:v>HSC_Curso sobre avaliação biológica ISO 10993_certificado-3533631.pdf</x:v>
+        <x:v>HSC_Curso sobre MDSAP AU_certificado-3533417.pdf</x:v>
       </x:c>
       <x:c r="B113" s="24" t="str">
         <x:v>PDF/imagem sem texto extraível</x:v>
@@ -15996,7 +16022,7 @@
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="24" t="str">
-        <x:v>HSC_Curso sobre Avaliação Clínica ISO 10993_certificado-3533419.pdf</x:v>
+        <x:v>HSC_ISO 10994 Gestão de Risco_certificado-3536529.pdf</x:v>
       </x:c>
       <x:c r="B114" s="24" t="str">
         <x:v>PDF/imagem sem texto extraível</x:v>
@@ -16011,7 +16037,7 @@
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="24" t="str">
-        <x:v>HSC_Curso sobre MDSAP AU_certificado-3533417.pdf</x:v>
+        <x:v>HSC_Registro no FDA_certificado-3533688.pdf</x:v>
       </x:c>
       <x:c r="B115" s="24" t="str">
         <x:v>PDF/imagem sem texto extraível</x:v>
@@ -16026,10 +16052,10 @@
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="24" t="str">
-        <x:v>HSC_ISO 10994 Gestão de Risco_certificado-3536529.pdf</x:v>
+        <x:v>HTH_Systems Thinking and Design Certificate.pdf</x:v>
       </x:c>
       <x:c r="B116" s="24" t="str">
-        <x:v>PDF/imagem sem texto extraível</x:v>
+        <x:v>Carga horária não localizada</x:v>
       </x:c>
       <x:c r="C116" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -16041,7 +16067,7 @@
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="24" t="str">
-        <x:v>HSC_Registro no FDA_certificado-3533688.pdf</x:v>
+        <x:v>IBSEC_ISO 27001 Essentials_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B117" s="24" t="str">
         <x:v>PDF/imagem sem texto extraível</x:v>
@@ -16056,10 +16082,10 @@
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="24" t="str">
-        <x:v>HTH_Systems Thinking and Design Certificate.pdf</x:v>
+        <x:v>IBSEC_ISO 27001 Fundamentos_ProfCertificate.pdf</x:v>
       </x:c>
       <x:c r="B118" s="24" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>PDF/imagem sem texto extraível</x:v>
       </x:c>
       <x:c r="C118" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -16071,7 +16097,7 @@
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="24" t="str">
-        <x:v>IBSEC_ISO 27001 Essentials_Certificate.pdf</x:v>
+        <x:v>IBSEC_Perícia Digital, Investigação e Custódia Segurança Digital_Essentials_ProfCertificate.pdf</x:v>
       </x:c>
       <x:c r="B119" s="24" t="str">
         <x:v>PDF/imagem sem texto extraível</x:v>
@@ -16086,10 +16112,10 @@
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="24" t="str">
-        <x:v>IBSEC_ISO 27001 Fundamentos_ProfCertificate.pdf</x:v>
+        <x:v>IIBA_6S Green Belt Certificate.pdf</x:v>
       </x:c>
       <x:c r="B120" s="24" t="str">
-        <x:v>PDF/imagem sem texto extraível</x:v>
+        <x:v>Carga horária não localizada</x:v>
       </x:c>
       <x:c r="C120" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -16101,7 +16127,7 @@
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="24" t="str">
-        <x:v>IBSEC_Perícia Digital, Investigação e Custódia Segurança Digital_Essentials_ProfCertificate.pdf</x:v>
+        <x:v>Injetáveis Curso_certificate_1779855229036 (1).pdf</x:v>
       </x:c>
       <x:c r="B121" s="24" t="str">
         <x:v>PDF/imagem sem texto extraível</x:v>
@@ -16116,10 +16142,10 @@
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="24" t="str">
-        <x:v>IIBA_6S Green Belt Certificate.pdf</x:v>
+        <x:v>Injetáveis Curso_certificate_1779855229036.pdf</x:v>
       </x:c>
       <x:c r="B122" s="24" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>PDF/imagem sem texto extraível</x:v>
       </x:c>
       <x:c r="C122" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -16131,10 +16157,10 @@
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="24" t="str">
-        <x:v>Injetáveis Curso_certificate_1779855229036 (1).pdf</x:v>
+        <x:v>International Institute of Business Analysis (IIBA®).pdf</x:v>
       </x:c>
       <x:c r="B123" s="24" t="str">
-        <x:v>PDF/imagem sem texto extraível</x:v>
+        <x:v>Carga horária não localizada</x:v>
       </x:c>
       <x:c r="C123" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -16146,7 +16172,7 @@
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="24" t="str">
-        <x:v>Injetáveis Curso_certificate_1779855229036.pdf</x:v>
+        <x:v>IPE-Creighton - Certicate-ish.docx</x:v>
       </x:c>
       <x:c r="B124" s="24" t="str">
         <x:v>PDF/imagem sem texto extraível</x:v>
@@ -16161,7 +16187,7 @@
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="24" t="str">
-        <x:v>International Institute of Business Analysis (IIBA®).pdf</x:v>
+        <x:v>ISO 9001 and 27001 Essentials Certificate_Great Learning.pdf</x:v>
       </x:c>
       <x:c r="B125" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16169,14 +16195,16 @@
       <x:c r="C125" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
       </x:c>
-      <x:c r="D125" s="24" t="str"/>
+      <x:c r="D125" s="24" t="str">
+        <x:v>https://www.mygreatlearning.com/certificate/PSXVKTXD</x:v>
+      </x:c>
       <x:c r="E125" s="24" t="str">
         <x:v>Pendente</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="24" t="str">
-        <x:v>IPE-Creighton - Certicate-ish.docx</x:v>
+        <x:v>ISO9001_Badge_SkillFront96337181584206.png</x:v>
       </x:c>
       <x:c r="B126" s="24" t="str">
         <x:v>PDF/imagem sem texto extraível</x:v>
@@ -16191,24 +16219,22 @@
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="24" t="str">
-        <x:v>ISO 9001 and 27001 Essentials Certificate_Great Learning.pdf</x:v>
+        <x:v>IU_Primary Plagiarism Certificate.pdf</x:v>
       </x:c>
       <x:c r="B127" s="24" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>PDF/imagem sem texto extraível</x:v>
       </x:c>
       <x:c r="C127" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
       </x:c>
-      <x:c r="D127" s="24" t="str">
-        <x:v>https://www.mygreatlearning.com/certificate/PSXVKTXD</x:v>
-      </x:c>
+      <x:c r="D127" s="24" t="str"/>
       <x:c r="E127" s="24" t="str">
         <x:v>Pendente</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="24" t="str">
-        <x:v>ISO9001_Badge_SkillFront96337181584206.png</x:v>
+        <x:v>IU_Primary Plagiarism Certificate_signed.pdf</x:v>
       </x:c>
       <x:c r="B128" s="24" t="str">
         <x:v>PDF/imagem sem texto extraível</x:v>
@@ -16223,10 +16249,10 @@
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="24" t="str">
-        <x:v>IU_Primary Plagiarism Certificate.pdf</x:v>
+        <x:v>LinkedIn Learning_Building Blocks in AI Certificate.pdf</x:v>
       </x:c>
       <x:c r="B129" s="24" t="str">
-        <x:v>PDF/imagem sem texto extraível</x:v>
+        <x:v>Carga horária não localizada</x:v>
       </x:c>
       <x:c r="C129" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -16238,10 +16264,10 @@
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="24" t="str">
-        <x:v>IU_Primary Plagiarism Certificate_signed.pdf</x:v>
+        <x:v>LinkedIn_AI para Profissionais da Justiça_Certificado.pdf</x:v>
       </x:c>
       <x:c r="B130" s="24" t="str">
-        <x:v>PDF/imagem sem texto extraível</x:v>
+        <x:v>Carga horária não localizada</x:v>
       </x:c>
       <x:c r="C130" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -16253,7 +16279,7 @@
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="24" t="str">
-        <x:v>JHU-Coursera_Biostatistics in PH_4XIVGLM9A4VF.pdf</x:v>
+        <x:v>LinkedIn_AI Products Introduction_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B131" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16268,7 +16294,7 @@
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="24" t="str">
-        <x:v>LinkedIn Learning_Building Blocks in AI Certificate.pdf</x:v>
+        <x:v>LinkedIn_Top Performers Reinvention_Completion Certificate.pdf</x:v>
       </x:c>
       <x:c r="B132" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16283,7 +16309,7 @@
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="24" t="str">
-        <x:v>LinkedIn_AI para Profissionais da Justiça_Certificado.pdf</x:v>
+        <x:v>LOC Certificate for 'Breaking the Routine- Modernizing Mealtime Insulin Manageme.pdf</x:v>
       </x:c>
       <x:c r="B133" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16298,10 +16324,10 @@
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="24" t="str">
-        <x:v>LinkedIn_AI Products Introduction_Certificate.pdf</x:v>
+        <x:v>MedScape_Updates on infections_LOC Certificate.pdf</x:v>
       </x:c>
       <x:c r="B134" s="24" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>PDF/imagem sem texto extraível</x:v>
       </x:c>
       <x:c r="C134" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -16313,7 +16339,7 @@
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="24" t="str">
-        <x:v>LinkedIn_Top Performers Reinvention_Completion Certificate.pdf</x:v>
+        <x:v>My Support Cases.pdf</x:v>
       </x:c>
       <x:c r="B135" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16321,14 +16347,16 @@
       <x:c r="C135" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
       </x:c>
-      <x:c r="D135" s="24" t="str"/>
+      <x:c r="D135" s="24" t="str">
+        <x:v>https://www.coursera.org/my-purchases/transactions?utm_medium=email&amp;utm_source=other&amp;utm_campaign=…</x:v>
+      </x:c>
       <x:c r="E135" s="24" t="str">
         <x:v>Pendente</x:v>
       </x:c>
     </x:row>
     <x:row r="136">
       <x:c r="A136" s="24" t="str">
-        <x:v>LOC Certificate for 'Breaking the Routine- Modernizing Mealtime Insulin Manageme.pdf</x:v>
+        <x:v>My Support Casespt2.pdf</x:v>
       </x:c>
       <x:c r="B136" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16336,17 +16364,19 @@
       <x:c r="C136" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
       </x:c>
-      <x:c r="D136" s="24" t="str"/>
+      <x:c r="D136" s="24" t="str">
+        <x:v>http://play.google.com/store/apps/details? | https://about.coursera.org/ | https://about.coursera.org/afﬁliates | https://about.coursera.org/careers | https://about.coursera.org/how-coursera-works/ | https://about.coursera.org/leadership | https://blog.coursera.org/ | https://building.coursera.org/developer-program/ | https://investor.coursera.com/ | https://itunes.apple.com/app/apple- | https://learner.coursera.help/hc | https://learner.coursera.help/hc/articles/360050668591- | https://medium.com/coursera-engineering | https://www.coursera.community/ | https://www.coursera.community/#beta-tester | https://www.coursera.community/#gtc | https://www.coursera.org/about/contact | https://www.coursera.org/about/partners | https://www.coursera.org/about/press | https://www.coursera.org/about/privacy | https://www.coursera.org/about/terms | https://www.coursera.org/articles | https://www.coursera.org/browse | https://www.coursera.org/business | https://www.coursera.org/campus | https://www.coursera.org/degrees | https://www.coursera.org/directory | https://www.coursera.org/government | https://www.coursera.org/professional- | https://www.coursera.org/teaching-center</x:v>
+      </x:c>
       <x:c r="E136" s="24" t="str">
         <x:v>Pendente</x:v>
       </x:c>
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="24" t="str">
-        <x:v>MedScape_Updates on infections_LOC Certificate.pdf</x:v>
+        <x:v>NASB-LinkedIn_Certificate_PME_Budgets.pdf</x:v>
       </x:c>
       <x:c r="B137" s="24" t="str">
-        <x:v>PDF/imagem sem texto extraível</x:v>
+        <x:v>Carga horária não localizada</x:v>
       </x:c>
       <x:c r="C137" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -16358,7 +16388,7 @@
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="24" t="str">
-        <x:v>My Support Cases.pdf</x:v>
+        <x:v>NASBA-LikedIn_PMF_Communication_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B138" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16366,16 +16396,14 @@
       <x:c r="C138" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
       </x:c>
-      <x:c r="D138" s="24" t="str">
-        <x:v>https://www.coursera.org/my-purchases/transactions?utm_medium=email&amp;utm_source=other&amp;utm_campaign=…</x:v>
-      </x:c>
+      <x:c r="D138" s="24" t="str"/>
       <x:c r="E138" s="24" t="str">
         <x:v>Pendente</x:v>
       </x:c>
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="24" t="str">
-        <x:v>My Support Casespt2.pdf</x:v>
+        <x:v>NASBA-LinkedIn Certificate - Six Sigma Black Belt.pdf</x:v>
       </x:c>
       <x:c r="B139" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16383,16 +16411,14 @@
       <x:c r="C139" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
       </x:c>
-      <x:c r="D139" s="24" t="str">
-        <x:v>http://play.google.com/store/apps/details? | https://about.coursera.org/ | https://about.coursera.org/afﬁliates | https://about.coursera.org/careers | https://about.coursera.org/how-coursera-works/ | https://about.coursera.org/leadership | https://blog.coursera.org/ | https://building.coursera.org/developer-program/ | https://investor.coursera.com/ | https://itunes.apple.com/app/apple- | https://learner.coursera.help/hc | https://learner.coursera.help/hc/articles/360050668591- | https://medium.com/coursera-engineering | https://www.coursera.community/ | https://www.coursera.community/#beta-tester | https://www.coursera.community/#gtc | https://www.coursera.org/about/contact | https://www.coursera.org/about/partners | https://www.coursera.org/about/press | https://www.coursera.org/about/privacy | https://www.coursera.org/about/terms | https://www.coursera.org/articles | https://www.coursera.org/browse | https://www.coursera.org/business | https://www.coursera.org/campus | https://www.coursera.org/degrees | https://www.coursera.org/directory | https://www.coursera.org/government | https://www.coursera.org/professional- | https://www.coursera.org/teaching-center</x:v>
-      </x:c>
+      <x:c r="D139" s="24" t="str"/>
       <x:c r="E139" s="24" t="str">
         <x:v>Pendente</x:v>
       </x:c>
     </x:row>
     <x:row r="140">
       <x:c r="A140" s="24" t="str">
-        <x:v>NASB-LinkedIn_Certificate_PME_Budgets.pdf</x:v>
+        <x:v>NASBA-LinkedIn Certificate_PMF_Teams.pdf</x:v>
       </x:c>
       <x:c r="B140" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16407,7 +16433,7 @@
     </x:row>
     <x:row r="141">
       <x:c r="A141" s="24" t="str">
-        <x:v>NASBA-LikedIn_PMF_Communication_Certificate.pdf</x:v>
+        <x:v>NASBA-LinkedIn Certificate_Project Management Foundations.pdf</x:v>
       </x:c>
       <x:c r="B141" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16422,7 +16448,7 @@
     </x:row>
     <x:row r="142">
       <x:c r="A142" s="24" t="str">
-        <x:v>NASBA-LinkedIn Certificate - Six Sigma Black Belt.pdf</x:v>
+        <x:v>NASBA-LinkedIn Learning - PM Risk Certificate.pdf</x:v>
       </x:c>
       <x:c r="B142" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16437,7 +16463,7 @@
     </x:row>
     <x:row r="143">
       <x:c r="A143" s="24" t="str">
-        <x:v>NASBA-LinkedIn Certificate_PMF_Teams.pdf</x:v>
+        <x:v>NASBA-LinkedIn_Certificate_PM Foundations_Ethics.pdf</x:v>
       </x:c>
       <x:c r="B143" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16452,7 +16478,7 @@
     </x:row>
     <x:row r="144">
       <x:c r="A144" s="24" t="str">
-        <x:v>NASBA-LinkedIn Certificate_Project Management Foundations.pdf</x:v>
+        <x:v>NASBA-LinkedIn_MicrosoftMPM_Certificaye.pdf</x:v>
       </x:c>
       <x:c r="B144" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16467,7 +16493,7 @@
     </x:row>
     <x:row r="145">
       <x:c r="A145" s="24" t="str">
-        <x:v>NASBA-LinkedIn Learning - PM Risk Certificate.pdf</x:v>
+        <x:v>NASBA-LinkedIn_PM Foundations Requirements.pdf</x:v>
       </x:c>
       <x:c r="B145" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16482,7 +16508,7 @@
     </x:row>
     <x:row r="146">
       <x:c r="A146" s="24" t="str">
-        <x:v>NASBA-LinkedIn_Certificate_PM Foundations_Ethics.pdf</x:v>
+        <x:v>NASBA-LinkedIn_PME_Schedules.pdf</x:v>
       </x:c>
       <x:c r="B146" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16497,7 +16523,7 @@
     </x:row>
     <x:row r="147">
       <x:c r="A147" s="24" t="str">
-        <x:v>NASBA-LinkedIn_MicrosoftMPM_Certificaye.pdf</x:v>
+        <x:v>NASBA-LinkedIn_PMF_Risks Certificate_.pdf</x:v>
       </x:c>
       <x:c r="B147" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16512,7 +16538,7 @@
     </x:row>
     <x:row r="148">
       <x:c r="A148" s="24" t="str">
-        <x:v>NASBA-LinkedIn_PM Foundations Requirements.pdf</x:v>
+        <x:v>NASBA-LinkedIn_PMF_Stakeholders_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B148" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16527,7 +16553,7 @@
     </x:row>
     <x:row r="149">
       <x:c r="A149" s="24" t="str">
-        <x:v>NASBA-LinkedIn_PME_Schedules.pdf</x:v>
+        <x:v>NASBA_Certificate_Healthcare Projects.pdf</x:v>
       </x:c>
       <x:c r="B149" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16542,7 +16568,7 @@
     </x:row>
     <x:row r="150">
       <x:c r="A150" s="24" t="str">
-        <x:v>NASBA-LinkedIn_PMF_Risks Certificate_.pdf</x:v>
+        <x:v>New opioid treatments_cmeucert_20260731_134129.pdf</x:v>
       </x:c>
       <x:c r="B150" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16557,7 +16583,7 @@
     </x:row>
     <x:row r="151">
       <x:c r="A151" s="24" t="str">
-        <x:v>NASBA-LinkedIn_PMF_Stakeholders_Certificate.pdf</x:v>
+        <x:v>NIDA GCP Certificate.pdf</x:v>
       </x:c>
       <x:c r="B151" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16572,10 +16598,10 @@
     </x:row>
     <x:row r="152">
       <x:c r="A152" s="24" t="str">
-        <x:v>NASBA_Certificate_Healthcare Projects.pdf</x:v>
+        <x:v>Pedro Lamounier Sampaio - CV 2.pdf</x:v>
       </x:c>
       <x:c r="B152" s="24" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>PDF/imagem sem texto extraível</x:v>
       </x:c>
       <x:c r="C152" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -16587,7 +16613,7 @@
     </x:row>
     <x:row r="153">
       <x:c r="A153" s="24" t="str">
-        <x:v>New opioid treatments_cmeucert_20260731_134129.pdf</x:v>
+        <x:v>Pedro Lamounier Sampaio - PDF Certificate (ISO 19011 Lead Auditor).pdf</x:v>
       </x:c>
       <x:c r="B153" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16602,10 +16628,10 @@
     </x:row>
     <x:row r="154">
       <x:c r="A154" s="24" t="str">
-        <x:v>NIDA GCP Certificate.pdf</x:v>
+        <x:v>Pedro Lamounier Sampaio _ LinkedIn_Duolingo LVL128.pdf</x:v>
       </x:c>
       <x:c r="B154" s="24" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>PDF/imagem sem texto extraível</x:v>
       </x:c>
       <x:c r="C154" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -16617,10 +16643,10 @@
     </x:row>
     <x:row r="155">
       <x:c r="A155" s="24" t="str">
-        <x:v>Pedro Lamounier Sampaio - CV 2.pdf</x:v>
+        <x:v>Pedro Lamounier Sampaio ACLS (Advanced Cardiac Life Support) Online Course Completion Certificate 2026.pdf</x:v>
       </x:c>
       <x:c r="B155" s="24" t="str">
-        <x:v>PDF/imagem sem texto extraível</x:v>
+        <x:v>Carga horária não localizada</x:v>
       </x:c>
       <x:c r="C155" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -16632,7 +16658,7 @@
     </x:row>
     <x:row r="156">
       <x:c r="A156" s="24" t="str">
-        <x:v>Pedro Lamounier Sampaio - PDF Certificate (ISO 19011 Lead Auditor).pdf</x:v>
+        <x:v>Pedro Lamounier Sampaio ACLS Course Completion Certificate.pdf</x:v>
       </x:c>
       <x:c r="B156" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16647,10 +16673,10 @@
     </x:row>
     <x:row r="157">
       <x:c r="A157" s="24" t="str">
-        <x:v>Pedro Lamounier Sampaio _ LinkedIn_Duolingo LVL128.pdf</x:v>
+        <x:v>Pedro Lamounier Sampaio BLS (Basic Life Support) Online Course Completion Certificate 2026.pdf</x:v>
       </x:c>
       <x:c r="B157" s="24" t="str">
-        <x:v>PDF/imagem sem texto extraível</x:v>
+        <x:v>Carga horária não localizada</x:v>
       </x:c>
       <x:c r="C157" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -16662,7 +16688,7 @@
     </x:row>
     <x:row r="158">
       <x:c r="A158" s="24" t="str">
-        <x:v>Pedro Lamounier Sampaio ACLS (Advanced Cardiac Life Support) Online Course Completion Certificate 2026.pdf</x:v>
+        <x:v>Pedro Lamounier Sampaio- PDF Certificate (Advanced Cardiac Life Support (ACLS)).pdf</x:v>
       </x:c>
       <x:c r="B158" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16677,10 +16703,10 @@
     </x:row>
     <x:row r="159">
       <x:c r="A159" s="24" t="str">
-        <x:v>Pedro Lamounier Sampaio ACLS Course Completion Certificate.pdf</x:v>
+        <x:v>PEDRO_LAMOUNIER_SAMPAIO_Cybersecurity_Awareness_-_Production.pdf</x:v>
       </x:c>
       <x:c r="B159" s="24" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>PDF/imagem sem texto extraível</x:v>
       </x:c>
       <x:c r="C159" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -16692,10 +16718,10 @@
     </x:row>
     <x:row r="160">
       <x:c r="A160" s="24" t="str">
-        <x:v>Pedro Lamounier Sampaio BLS (Basic Life Support) Online Course Completion Certificate 2026.pdf</x:v>
+        <x:v>PEDRO_LAMOUNIER_SAMPAIO_Project_Management_Essentials_-_Production.pdf</x:v>
       </x:c>
       <x:c r="B160" s="24" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>PDF/imagem sem texto extraível</x:v>
       </x:c>
       <x:c r="C160" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -16707,7 +16733,7 @@
     </x:row>
     <x:row r="161">
       <x:c r="A161" s="24" t="str">
-        <x:v>Pedro Lamounier Sampaio- PDF Certificate (Advanced Cardiac Life Support (ACLS)).pdf</x:v>
+        <x:v>Personalidade INTP (Lógico) _ 16Personalities.pdf</x:v>
       </x:c>
       <x:c r="B161" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16722,7 +16748,7 @@
     </x:row>
     <x:row r="162">
       <x:c r="A162" s="24" t="str">
-        <x:v>PEDRO_LAMOUNIER_SAMPAIO_Cybersecurity_Awareness_-_Production.pdf</x:v>
+        <x:v>PET_ESOL Entry 3 Certificate.pdf</x:v>
       </x:c>
       <x:c r="B162" s="24" t="str">
         <x:v>PDF/imagem sem texto extraível</x:v>
@@ -16737,10 +16763,10 @@
     </x:row>
     <x:row r="163">
       <x:c r="A163" s="24" t="str">
-        <x:v>PEDRO_LAMOUNIER_SAMPAIO_Project_Management_Essentials_-_Production.pdf</x:v>
+        <x:v>PHC Course - WHO Academy.pdf</x:v>
       </x:c>
       <x:c r="B163" s="24" t="str">
-        <x:v>PDF/imagem sem texto extraível</x:v>
+        <x:v>Carga horária não localizada</x:v>
       </x:c>
       <x:c r="C163" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -16752,7 +16778,7 @@
     </x:row>
     <x:row r="164">
       <x:c r="A164" s="24" t="str">
-        <x:v>Personalidade INTP (Lógico) _ 16Personalities.pdf</x:v>
+        <x:v>pjrtraining _ ISO 9001-2015 Clause-by-Clau... (CBC9000) _ Final Exam.pdf</x:v>
       </x:c>
       <x:c r="B164" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16760,17 +16786,19 @@
       <x:c r="C164" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
       </x:c>
-      <x:c r="D164" s="24" t="str"/>
+      <x:c r="D164" s="24" t="str">
+        <x:v>https://pjrtraining.talentlms.com/dashboard | https://pjrtraining.talentlms.com/unit/viewtestsurvey/id:1746,mode:test</x:v>
+      </x:c>
       <x:c r="E164" s="24" t="str">
         <x:v>Pendente</x:v>
       </x:c>
     </x:row>
     <x:row r="165">
       <x:c r="A165" s="24" t="str">
-        <x:v>PET_ESOL Entry 3 Certificate.pdf</x:v>
+        <x:v>PMI-LinkedIn Certificate - Six Sigma Black Belt.pdf</x:v>
       </x:c>
       <x:c r="B165" s="24" t="str">
-        <x:v>PDF/imagem sem texto extraível</x:v>
+        <x:v>Carga horária não localizada</x:v>
       </x:c>
       <x:c r="C165" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -16782,7 +16810,7 @@
     </x:row>
     <x:row r="166">
       <x:c r="A166" s="24" t="str">
-        <x:v>PHC Course - WHO Academy.pdf</x:v>
+        <x:v>PMI-LinkedIn Certificate_Problem Solving for Leadership.pdf</x:v>
       </x:c>
       <x:c r="B166" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16797,7 +16825,7 @@
     </x:row>
     <x:row r="167">
       <x:c r="A167" s="24" t="str">
-        <x:v>pjrtraining _ ISO 9001-2015 Clause-by-Clau... (CBC9000) _ Final Exam.pdf</x:v>
+        <x:v>PMI-LinkedIn Certificate_Project Management Foundations.pdf</x:v>
       </x:c>
       <x:c r="B167" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16805,16 +16833,14 @@
       <x:c r="C167" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
       </x:c>
-      <x:c r="D167" s="24" t="str">
-        <x:v>https://pjrtraining.talentlms.com/dashboard | https://pjrtraining.talentlms.com/unit/viewtestsurvey/id:1746,mode:test</x:v>
-      </x:c>
+      <x:c r="D167" s="24" t="str"/>
       <x:c r="E167" s="24" t="str">
         <x:v>Pendente</x:v>
       </x:c>
     </x:row>
     <x:row r="168">
       <x:c r="A168" s="24" t="str">
-        <x:v>PMI-LinkedIn Certificate - Six Sigma Black Belt.pdf</x:v>
+        <x:v>PMI-LinkedIn Learning Certificate_Healthcare Projects.pdf</x:v>
       </x:c>
       <x:c r="B168" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16829,7 +16855,7 @@
     </x:row>
     <x:row r="169">
       <x:c r="A169" s="24" t="str">
-        <x:v>PMI-LinkedIn Certificate_Problem Solving for Leadership.pdf</x:v>
+        <x:v>PMI-LinkedIn_Certificate_PM Foundations Requirements.pdf</x:v>
       </x:c>
       <x:c r="B169" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16844,7 +16870,7 @@
     </x:row>
     <x:row r="170">
       <x:c r="A170" s="24" t="str">
-        <x:v>PMI-LinkedIn Certificate_Project Management Foundations.pdf</x:v>
+        <x:v>PMI-LinkedIn_Certificate_PM Foundations_Ethics.pdf</x:v>
       </x:c>
       <x:c r="B170" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16859,7 +16885,7 @@
     </x:row>
     <x:row r="171">
       <x:c r="A171" s="24" t="str">
-        <x:v>PMI-LinkedIn Learning Certificate_Healthcare Projects.pdf</x:v>
+        <x:v>PMI-LinkedIn_Certificate_PME_Budgets.pdf</x:v>
       </x:c>
       <x:c r="B171" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16874,7 +16900,7 @@
     </x:row>
     <x:row r="172">
       <x:c r="A172" s="24" t="str">
-        <x:v>PMI-LinkedIn_Certificate_PM Foundations Requirements.pdf</x:v>
+        <x:v>PMI-LinkedIn_Certificate_PME_Schedules.pdf</x:v>
       </x:c>
       <x:c r="B172" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16889,7 +16915,7 @@
     </x:row>
     <x:row r="173">
       <x:c r="A173" s="24" t="str">
-        <x:v>PMI-LinkedIn_Certificate_PM Foundations_Ethics.pdf</x:v>
+        <x:v>PMI-LinkedIn_Certificate_PMF_Teams.pdf</x:v>
       </x:c>
       <x:c r="B173" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16904,7 +16930,7 @@
     </x:row>
     <x:row r="174">
       <x:c r="A174" s="24" t="str">
-        <x:v>PMI-LinkedIn_Certificate_PME_Budgets.pdf</x:v>
+        <x:v>PMI-LinkedIn_Leveraging AI_GRC_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B174" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16919,7 +16945,7 @@
     </x:row>
     <x:row r="175">
       <x:c r="A175" s="24" t="str">
-        <x:v>PMI-LinkedIn_Certificate_PME_Schedules.pdf</x:v>
+        <x:v>PMI-LinkedIn_MicrosoftMPM_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B175" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16934,7 +16960,7 @@
     </x:row>
     <x:row r="176">
       <x:c r="A176" s="24" t="str">
-        <x:v>PMI-LinkedIn_Certificate_PMF_Teams.pdf</x:v>
+        <x:v>PMI-LinkedIn_PMF_Communication_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B176" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16949,7 +16975,7 @@
     </x:row>
     <x:row r="177">
       <x:c r="A177" s="24" t="str">
-        <x:v>PMI-LinkedIn_Leveraging AI_GRC_Certificate.pdf</x:v>
+        <x:v>PMI-LinkedIn_PMF_Risks_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B177" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16964,7 +16990,7 @@
     </x:row>
     <x:row r="178">
       <x:c r="A178" s="24" t="str">
-        <x:v>PMI-LinkedIn_MicrosoftMPM_Certificate.pdf</x:v>
+        <x:v>PMI-LinkedIn_PMF_Stakeholders_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B178" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16979,7 +17005,7 @@
     </x:row>
     <x:row r="179">
       <x:c r="A179" s="24" t="str">
-        <x:v>PMI-LinkedIn_PMF_Communication_Certificate.pdf</x:v>
+        <x:v>PMI_LinkedIn_Certificate_AI_Projects.pdf</x:v>
       </x:c>
       <x:c r="B179" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -16994,7 +17020,7 @@
     </x:row>
     <x:row r="180">
       <x:c r="A180" s="24" t="str">
-        <x:v>PMI-LinkedIn_PMF_Risks_Certificate.pdf</x:v>
+        <x:v>PMP ExamPrep1_Project Management Institute (PMI)®.pdf</x:v>
       </x:c>
       <x:c r="B180" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -17009,7 +17035,7 @@
     </x:row>
     <x:row r="181">
       <x:c r="A181" s="24" t="str">
-        <x:v>PMI-LinkedIn_PMF_Stakeholders_Certificate.pdf</x:v>
+        <x:v>Podcast APS_CME answers certificate-2026-7-12_1735.pdf</x:v>
       </x:c>
       <x:c r="B181" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -17017,14 +17043,16 @@
       <x:c r="C181" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
       </x:c>
-      <x:c r="D181" s="24" t="str"/>
+      <x:c r="D181" s="24" t="str">
+        <x:v>https://answersincme.com/DDT</x:v>
+      </x:c>
       <x:c r="E181" s="24" t="str">
         <x:v>Pendente</x:v>
       </x:c>
     </x:row>
     <x:row r="182">
       <x:c r="A182" s="24" t="str">
-        <x:v>PMI_LinkedIn_Certificate_AI_Projects.pdf</x:v>
+        <x:v>Processo Civil no pós-pandemia - Certificado ESAOAB.pdf</x:v>
       </x:c>
       <x:c r="B182" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -17039,7 +17067,7 @@
     </x:row>
     <x:row r="183">
       <x:c r="A183" s="24" t="str">
-        <x:v>PMP ExamPrep1_Project Management Institute (PMI)®.pdf</x:v>
+        <x:v>Project Management Institute (PMI)_6S Green Belt.pdf</x:v>
       </x:c>
       <x:c r="B183" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -17054,7 +17082,7 @@
     </x:row>
     <x:row r="184">
       <x:c r="A184" s="24" t="str">
-        <x:v>Podcast APS_CME answers certificate-2026-7-12_1735.pdf</x:v>
+        <x:v>Project Management Institute (PMI)®.pdf</x:v>
       </x:c>
       <x:c r="B184" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -17062,16 +17090,14 @@
       <x:c r="C184" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
       </x:c>
-      <x:c r="D184" s="24" t="str">
-        <x:v>https://answersincme.com/DDT</x:v>
-      </x:c>
+      <x:c r="D184" s="24" t="str"/>
       <x:c r="E184" s="24" t="str">
         <x:v>Pendente</x:v>
       </x:c>
     </x:row>
     <x:row r="185">
       <x:c r="A185" s="24" t="str">
-        <x:v>Processo Civil no pós-pandemia - Certificado ESAOAB.pdf</x:v>
+        <x:v>Public Health Law Academy_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B185" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -17086,10 +17112,10 @@
     </x:row>
     <x:row r="186">
       <x:c r="A186" s="24" t="str">
-        <x:v>Project Management Institute (PMI)_6S Green Belt.pdf</x:v>
+        <x:v>Python.pdf</x:v>
       </x:c>
       <x:c r="B186" s="24" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>PDF/imagem sem texto extraível</x:v>
       </x:c>
       <x:c r="C186" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -17101,7 +17127,7 @@
     </x:row>
     <x:row r="187">
       <x:c r="A187" s="24" t="str">
-        <x:v>Project Management Institute (PMI)®.pdf</x:v>
+        <x:v>QMS_ISO 19011-2026_Fundamentos_Certificado 0014912.pdf</x:v>
       </x:c>
       <x:c r="B187" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -17116,7 +17142,7 @@
     </x:row>
     <x:row r="188">
       <x:c r="A188" s="24" t="str">
-        <x:v>Public Health Law Academy_Certificate.pdf</x:v>
+        <x:v>Relatório_Extensao_CEPROC.pdf</x:v>
       </x:c>
       <x:c r="B188" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -17131,10 +17157,10 @@
     </x:row>
     <x:row r="189">
       <x:c r="A189" s="24" t="str">
-        <x:v>Python.pdf</x:v>
+        <x:v>revivr-CPR_certificate_2026.08.22.pdf</x:v>
       </x:c>
       <x:c r="B189" s="24" t="str">
-        <x:v>PDF/imagem sem texto extraível</x:v>
+        <x:v>Carga horária não localizada</x:v>
       </x:c>
       <x:c r="C189" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -17146,7 +17172,7 @@
     </x:row>
     <x:row r="190">
       <x:c r="A190" s="24" t="str">
-        <x:v>QMS_ISO 19011-2026_Fundamentos_Certificado 0014912.pdf</x:v>
+        <x:v>SkillFront-ISO 9001_Associate_Certificate_SFE0232f5d549bbc-96337181584206.pdf</x:v>
       </x:c>
       <x:c r="B190" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -17161,7 +17187,7 @@
     </x:row>
     <x:row r="191">
       <x:c r="A191" s="24" t="str">
-        <x:v>Relatório_Extensao_CEPROC.pdf</x:v>
+        <x:v>SkillFront_ISO 27001 ISMS Associate SFE0166da11827fd-47327192991292_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B191" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -17176,7 +17202,7 @@
     </x:row>
     <x:row r="192">
       <x:c r="A192" s="24" t="str">
-        <x:v>revivr-CPR_certificate_2026.08.22.pdf</x:v>
+        <x:v>texto 2.txt</x:v>
       </x:c>
       <x:c r="B192" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -17191,7 +17217,7 @@
     </x:row>
     <x:row r="193">
       <x:c r="A193" s="24" t="str">
-        <x:v>Said-Oxford-Coursera_Specialization AI for Business_Certificate_FWGA4AWODSM4.pdf</x:v>
+        <x:v>texto 3.txt</x:v>
       </x:c>
       <x:c r="B193" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -17199,14 +17225,16 @@
       <x:c r="C193" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
       </x:c>
-      <x:c r="D193" s="24" t="str"/>
+      <x:c r="D193" s="24" t="str">
+        <x:v>https://produto.mercadolivre.com.br/MLB-3554868073-creme-despigmentante-alfa-arbutin-7-40g-_JM", | https://shopee.com.br/search?keyword=Alfa+Arbutin+Axilas", | https://shopee.com.br/search?keyword=Alfa+Arbutin+Formulab", | https://shopee.com.br/search?keyword=Alfa+Arbutin+Locao", | https://shopee.com.br/search?keyword=Alpha+Arbutin", | https://shopee.com.br/search?keyword=Creme%20Gel%20para%20Peeling%20com%20%C3%81cido%20Retin%C3%B3ico%20e%20Hidroquinona", | https://shopee.com.br/search?keyword=Hidroquinona", | https://www.amazon.com.br/alpha-arbutin/s?k=alpha+arbutin", | https://www.amazon.com.br/s?k=Gel+Facial+Alfa+Arbutin", | https://www.belezasaude.com.br/creme-alfa-arbutin-10-vitamina-c-estabilizada-10-40g", | https://www.drogariaminasbrasil.com.br/hidroquinona-5-acid-retinoico-0-025-dexametasona-0-05-creme-30g.html", | https://www.drogariaminasbrasil.com.br/search?q=hidroquinona", | https://www.drogariasaopaulo.com.br/search?w=Melan-Off", | https://www.drogariasaopaulo.com.br/search?w=suavicid", | https://www.drogasil.com.br/search?w=Blancy", | https://www.drogasil.com.br/search?w=Classis%20TX", | https://www.drogasil.com.br/search?w=vitacid%20plus", | https://www.epocacosmeticos.com.br/search?q=Eucerin+Anti+Pigment", | https://www.farmaciabelladona.com.br/search?q=alfa+arbutin", | https://www.farmaciabelladona.com.br/search?q=hidroquinona", | https://www.farmaciabotanica.com.br/search?q=alfa+arbutin", | https://www.farmaciaeficacia.com.br/search?q=alfa+arbutin", | https://www.farmaciaeficacia.com.br/search?q=hidroquinona", | https://www.farmasesi.com.br/produto/5424-hidroquinona--ems-400mg-4-creme-30g", | https://www.farmasite.com.br/hidroquinona-4-alfa-bisabolol-1-creme-30g", | https://www.farmasite.com.br/search?q=hidroquinona", | https://www.manipulart.com.br/search?q=hidroquinona" | https://www.manipulart.com.br/search?q=hidroquinona", | https://www.mercadolivre.com.br/p/MLB39792525", | https://www.mercadolivre.com.br/search?keyword=Arbutin+Creme", | https://www.mercadolivre.com.br/search?keyword=Raavi%20Alfa%20Arbutin", | https://www.naturalforma.com.br/search?q=alfa+arbutin", | https://www.naturalforma.com.br/search?q=hidroquinona", | https://www.panvel.com/search?q=hormoskin", | https://www.rituaria.com.br/produtos/formula-uniformizadora",</x:v>
+      </x:c>
       <x:c r="E193" s="24" t="str">
         <x:v>Pendente</x:v>
       </x:c>
     </x:row>
     <x:row r="194">
       <x:c r="A194" s="24" t="str">
-        <x:v>SkillFront-ISO 9001_Associate_Certificate_SFE0232f5d549bbc-96337181584206.pdf</x:v>
+        <x:v>texto.txt</x:v>
       </x:c>
       <x:c r="B194" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -17214,14 +17242,16 @@
       <x:c r="C194" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
       </x:c>
-      <x:c r="D194" s="24" t="str"/>
+      <x:c r="D194" s="24" t="str">
+        <x:v>https://cursa.app/pt/downapp</x:v>
+      </x:c>
       <x:c r="E194" s="24" t="str">
         <x:v>Pendente</x:v>
       </x:c>
     </x:row>
     <x:row r="195">
       <x:c r="A195" s="24" t="str">
-        <x:v>SkillFront_ISO 27001 ISMS Associate SFE0166da11827fd-47327192991292_Certificate.pdf</x:v>
+        <x:v>TRREE (2023)_Certificate of completion for module 1_Intro to Research.pdf</x:v>
       </x:c>
       <x:c r="B195" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -17229,14 +17259,16 @@
       <x:c r="C195" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
       </x:c>
-      <x:c r="D195" s="24" t="str"/>
+      <x:c r="D195" s="24" t="str">
+        <x:v>http://www.cihr-irsc.gc.ca/e/2891.html</x:v>
+      </x:c>
       <x:c r="E195" s="24" t="str">
         <x:v>Pendente</x:v>
       </x:c>
     </x:row>
     <x:row r="196">
       <x:c r="A196" s="24" t="str">
-        <x:v>texto 2.txt</x:v>
+        <x:v>TRREE (2023)_Certificate of completion for module 2_Ethics Evaluation in Research.pdf</x:v>
       </x:c>
       <x:c r="B196" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -17244,14 +17276,16 @@
       <x:c r="C196" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
       </x:c>
-      <x:c r="D196" s="24" t="str"/>
+      <x:c r="D196" s="24" t="str">
+        <x:v>http://www.cihr-irsc.gc.ca/e/2891.html</x:v>
+      </x:c>
       <x:c r="E196" s="24" t="str">
         <x:v>Pendente</x:v>
       </x:c>
     </x:row>
     <x:row r="197">
       <x:c r="A197" s="24" t="str">
-        <x:v>texto 3.txt</x:v>
+        <x:v>TRREE (2023)_Certificate of completion for module 3_Informed Consent_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B197" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -17260,7 +17294,7 @@
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
       </x:c>
       <x:c r="D197" s="24" t="str">
-        <x:v>https://produto.mercadolivre.com.br/MLB-3554868073-creme-despigmentante-alfa-arbutin-7-40g-_JM", | https://shopee.com.br/search?keyword=Alfa+Arbutin+Axilas", | https://shopee.com.br/search?keyword=Alfa+Arbutin+Formulab", | https://shopee.com.br/search?keyword=Alfa+Arbutin+Locao", | https://shopee.com.br/search?keyword=Alpha+Arbutin", | https://shopee.com.br/search?keyword=Creme%20Gel%20para%20Peeling%20com%20%C3%81cido%20Retin%C3%B3ico%20e%20Hidroquinona", | https://shopee.com.br/search?keyword=Hidroquinona", | https://www.amazon.com.br/alpha-arbutin/s?k=alpha+arbutin", | https://www.amazon.com.br/s?k=Gel+Facial+Alfa+Arbutin", | https://www.belezasaude.com.br/creme-alfa-arbutin-10-vitamina-c-estabilizada-10-40g", | https://www.drogariaminasbrasil.com.br/hidroquinona-5-acid-retinoico-0-025-dexametasona-0-05-creme-30g.html", | https://www.drogariaminasbrasil.com.br/search?q=hidroquinona", | https://www.drogariasaopaulo.com.br/search?w=Melan-Off", | https://www.drogariasaopaulo.com.br/search?w=suavicid", | https://www.drogasil.com.br/search?w=Blancy", | https://www.drogasil.com.br/search?w=Classis%20TX", | https://www.drogasil.com.br/search?w=vitacid%20plus", | https://www.epocacosmeticos.com.br/search?q=Eucerin+Anti+Pigment", | https://www.farmaciabelladona.com.br/search?q=alfa+arbutin", | https://www.farmaciabelladona.com.br/search?q=hidroquinona", | https://www.farmaciabotanica.com.br/search?q=alfa+arbutin", | https://www.farmaciaeficacia.com.br/search?q=alfa+arbutin", | https://www.farmaciaeficacia.com.br/search?q=hidroquinona", | https://www.farmasesi.com.br/produto/5424-hidroquinona--ems-400mg-4-creme-30g", | https://www.farmasite.com.br/hidroquinona-4-alfa-bisabolol-1-creme-30g", | https://www.farmasite.com.br/search?q=hidroquinona", | https://www.manipulart.com.br/search?q=hidroquinona" | https://www.manipulart.com.br/search?q=hidroquinona", | https://www.mercadolivre.com.br/p/MLB39792525", | https://www.mercadolivre.com.br/search?keyword=Arbutin+Creme", | https://www.mercadolivre.com.br/search?keyword=Raavi%20Alfa%20Arbutin", | https://www.naturalforma.com.br/search?q=alfa+arbutin", | https://www.naturalforma.com.br/search?q=hidroquinona", | https://www.panvel.com/search?q=hormoskin", | https://www.rituaria.com.br/produtos/formula-uniformizadora",</x:v>
+        <x:v>http://www.cihr-irsc.gc.ca/e/2891.html</x:v>
       </x:c>
       <x:c r="E197" s="24" t="str">
         <x:v>Pendente</x:v>
@@ -17268,7 +17302,7 @@
     </x:row>
     <x:row r="198">
       <x:c r="A198" s="24" t="str">
-        <x:v>texto.txt</x:v>
+        <x:v>TRREE_Module 4_R3_GCP_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B198" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -17277,7 +17311,7 @@
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
       </x:c>
       <x:c r="D198" s="24" t="str">
-        <x:v>https://cursa.app/pt/downapp</x:v>
+        <x:v>http://www.cihr-irsc.gc.ca/e/2891.html</x:v>
       </x:c>
       <x:c r="E198" s="24" t="str">
         <x:v>Pendente</x:v>
@@ -17285,7 +17319,7 @@
     </x:row>
     <x:row r="199">
       <x:c r="A199" s="24" t="str">
-        <x:v>TRREE (2023)_Certificate of completion for module 1_Intro to Research.pdf</x:v>
+        <x:v>TRREE_Module 4R2_GCP_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B199" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -17302,7 +17336,7 @@
     </x:row>
     <x:row r="200">
       <x:c r="A200" s="24" t="str">
-        <x:v>TRREE (2023)_Certificate of completion for module 2_Ethics Evaluation in Research.pdf</x:v>
+        <x:v>TRREE_Module 5.1 HIV Vaccine TrialsTraining certificate.pdf</x:v>
       </x:c>
       <x:c r="B200" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -17319,7 +17353,7 @@
     </x:row>
     <x:row r="201">
       <x:c r="A201" s="24" t="str">
-        <x:v>TRREE (2023)_Certificate of completion for module 3_Informed Consent_Certificate.pdf</x:v>
+        <x:v>TRREE_Module 5.2_Adolescent participants in HIV Trials_Training certificate - Module 5.2.pdf</x:v>
       </x:c>
       <x:c r="B201" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -17336,7 +17370,7 @@
     </x:row>
     <x:row r="202">
       <x:c r="A202" s="24" t="str">
-        <x:v>TRREE_Module 4_R3_GCP_Certificate.pdf</x:v>
+        <x:v>TRREE_Module 5.3_Ethics in PH Research_Training Certificate.pdf</x:v>
       </x:c>
       <x:c r="B202" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -17353,7 +17387,7 @@
     </x:row>
     <x:row r="203">
       <x:c r="A203" s="24" t="str">
-        <x:v>TRREE_Module 4R2_GCP_Certificate.pdf</x:v>
+        <x:v>TRREE_Reg. Frameworks_Suisse-2025_Certificate.pdf</x:v>
       </x:c>
       <x:c r="B203" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -17370,24 +17404,22 @@
     </x:row>
     <x:row r="204">
       <x:c r="A204" s="24" t="str">
-        <x:v>TRREE_Module 5.1 HIV Vaccine TrialsTraining certificate.pdf</x:v>
+        <x:v>UFMA_DRC na APS_Certificafdo de Curso.pdf</x:v>
       </x:c>
       <x:c r="B204" s="24" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>PDF/imagem sem texto extraível</x:v>
       </x:c>
       <x:c r="C204" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
       </x:c>
-      <x:c r="D204" s="24" t="str">
-        <x:v>http://www.cihr-irsc.gc.ca/e/2891.html</x:v>
-      </x:c>
+      <x:c r="D204" s="24" t="str"/>
       <x:c r="E204" s="24" t="str">
         <x:v>Pendente</x:v>
       </x:c>
     </x:row>
     <x:row r="205">
       <x:c r="A205" s="24" t="str">
-        <x:v>TRREE_Module 5.2_Adolescent participants in HIV Trials_Training certificate - Module 5.2.pdf</x:v>
+        <x:v>UFMG-UNA-SUS_M1_Atributos da APS_certificado_1f198775-dbe8-6290-b71e-85b8bf09b5ac.pdf</x:v>
       </x:c>
       <x:c r="B205" s="24" t="str">
         <x:v>Carga horária não localizada</x:v>
@@ -17395,50 +17427,44 @@
       <x:c r="C205" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
       </x:c>
-      <x:c r="D205" s="24" t="str">
-        <x:v>http://www.cihr-irsc.gc.ca/e/2891.html</x:v>
-      </x:c>
+      <x:c r="D205" s="24" t="str"/>
       <x:c r="E205" s="24" t="str">
         <x:v>Pendente</x:v>
       </x:c>
     </x:row>
     <x:row r="206">
       <x:c r="A206" s="24" t="str">
-        <x:v>TRREE_Module 5.3_Ethics in PH Research_Training Certificate.pdf</x:v>
+        <x:v>UNA-SUS-UFMA_Aperfeiçoamento em DRC_Certificado.pdf</x:v>
       </x:c>
       <x:c r="B206" s="24" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>PDF/imagem sem texto extraível</x:v>
       </x:c>
       <x:c r="C206" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
       </x:c>
-      <x:c r="D206" s="24" t="str">
-        <x:v>http://www.cihr-irsc.gc.ca/e/2891.html</x:v>
-      </x:c>
+      <x:c r="D206" s="24" t="str"/>
       <x:c r="E206" s="24" t="str">
         <x:v>Pendente</x:v>
       </x:c>
     </x:row>
     <x:row r="207">
       <x:c r="A207" s="24" t="str">
-        <x:v>TRREE_Reg. Frameworks_Suisse-2025_Certificate.pdf</x:v>
+        <x:v>UNA-SUS-UFMA_Atendimento Interdisciplinar DRC_M5_Certificado.pdf</x:v>
       </x:c>
       <x:c r="B207" s="24" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>PDF/imagem sem texto extraível</x:v>
       </x:c>
       <x:c r="C207" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
       </x:c>
-      <x:c r="D207" s="24" t="str">
-        <x:v>http://www.cihr-irsc.gc.ca/e/2891.html</x:v>
-      </x:c>
+      <x:c r="D207" s="24" t="str"/>
       <x:c r="E207" s="24" t="str">
         <x:v>Pendente</x:v>
       </x:c>
     </x:row>
     <x:row r="208">
       <x:c r="A208" s="24" t="str">
-        <x:v>UFMA_DRC na APS_Certificafdo de Curso.pdf</x:v>
+        <x:v>UNA-SUS-UFMA_Diálise Peritoneal_M4_Certificado.pdf</x:v>
       </x:c>
       <x:c r="B208" s="24" t="str">
         <x:v>PDF/imagem sem texto extraível</x:v>
@@ -17453,10 +17479,10 @@
     </x:row>
     <x:row r="209">
       <x:c r="A209" s="24" t="str">
-        <x:v>UFMG-UNA-SUS_M1_Atributos da APS_certificado_1f198775-dbe8-6290-b71e-85b8bf09b5ac.pdf</x:v>
+        <x:v>UNA-SUS-UFMA_IA na Saúde_Extensão_Certificado.pdf</x:v>
       </x:c>
       <x:c r="B209" s="24" t="str">
-        <x:v>Carga horária não localizada</x:v>
+        <x:v>PDF/imagem sem texto extraível</x:v>
       </x:c>
       <x:c r="C209" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -17468,7 +17494,7 @@
     </x:row>
     <x:row r="210">
       <x:c r="A210" s="24" t="str">
-        <x:v>UNA-SUS-UFMA_Aperfeiçoamento em DRC_Certificado.pdf</x:v>
+        <x:v>UNA-SUS-UFMA_Introdução à DRC_M1_Certificado.pdf</x:v>
       </x:c>
       <x:c r="B210" s="24" t="str">
         <x:v>PDF/imagem sem texto extraível</x:v>
@@ -17483,7 +17509,7 @@
     </x:row>
     <x:row r="211">
       <x:c r="A211" s="24" t="str">
-        <x:v>UNA-SUS-UFMA_Atendimento Interdisciplinar DRC_M5_Certificado.pdf</x:v>
+        <x:v>UNA-SUS-UFMA_Manejo clínico da DRC_M3_Certificado.pdf</x:v>
       </x:c>
       <x:c r="B211" s="24" t="str">
         <x:v>PDF/imagem sem texto extraível</x:v>
@@ -17498,7 +17524,7 @@
     </x:row>
     <x:row r="212">
       <x:c r="A212" s="24" t="str">
-        <x:v>UNA-SUS-UFMA_Diálise Peritoneal_M4_Certificado.pdf</x:v>
+        <x:v>UNA-SUS-UFMA_Registros e Qualidade na Saúde Digital_Certificado de Conclusao_.pdf</x:v>
       </x:c>
       <x:c r="B212" s="24" t="str">
         <x:v>PDF/imagem sem texto extraível</x:v>
@@ -17513,7 +17539,7 @@
     </x:row>
     <x:row r="213">
       <x:c r="A213" s="24" t="str">
-        <x:v>UNA-SUS-UFMA_IA na Saúde_Extensão_Certificado.pdf</x:v>
+        <x:v>UNA-SUS-UFMA_Saude Digital e SUS_Certificado Extensão.pdf</x:v>
       </x:c>
       <x:c r="B213" s="24" t="str">
         <x:v>PDF/imagem sem texto extraível</x:v>
@@ -17528,7 +17554,7 @@
     </x:row>
     <x:row r="214">
       <x:c r="A214" s="24" t="str">
-        <x:v>UNA-SUS-UFMA_Introdução à DRC_M1_Certificado.pdf</x:v>
+        <x:v>UNA-SUS-UFMA_Saúde Digital Inclusiva_Certificado.pdf</x:v>
       </x:c>
       <x:c r="B214" s="24" t="str">
         <x:v>PDF/imagem sem texto extraível</x:v>
@@ -17543,7 +17569,7 @@
     </x:row>
     <x:row r="215">
       <x:c r="A215" s="24" t="str">
-        <x:v>UNA-SUS-UFMA_Manejo clínico da DRC_M3_Certificado.pdf</x:v>
+        <x:v>UNA-SUS-UFMA_Saúde Digital Noções fundamentais_Certificado.pdf</x:v>
       </x:c>
       <x:c r="B215" s="24" t="str">
         <x:v>PDF/imagem sem texto extraível</x:v>
@@ -17558,7 +17584,7 @@
     </x:row>
     <x:row r="216">
       <x:c r="A216" s="24" t="str">
-        <x:v>UNA-SUS-UFMA_Registros e Qualidade na Saúde Digital_Certificado de Conclusao_.pdf</x:v>
+        <x:v>UNA-SUS-UFMA_Transf Digital_Extensao_Certificado.pdf</x:v>
       </x:c>
       <x:c r="B216" s="24" t="str">
         <x:v>PDF/imagem sem texto extraível</x:v>
@@ -17573,7 +17599,7 @@
     </x:row>
     <x:row r="217">
       <x:c r="A217" s="24" t="str">
-        <x:v>UNA-SUS-UFMA_Saude Digital e SUS_Certificado Extensão.pdf</x:v>
+        <x:v>UNA-SUS_Certificado_Introducao Saúde Digital.pdf</x:v>
       </x:c>
       <x:c r="B217" s="24" t="str">
         <x:v>PDF/imagem sem texto extraível</x:v>
@@ -17588,7 +17614,7 @@
     </x:row>
     <x:row r="218">
       <x:c r="A218" s="24" t="str">
-        <x:v>UNA-SUS-UFMA_Saúde Digital Inclusiva_Certificado.pdf</x:v>
+        <x:v>UNA-SUS_UFMA_Cultura da Saúde Digital_Certificado de Extensão_.pdf</x:v>
       </x:c>
       <x:c r="B218" s="24" t="str">
         <x:v>PDF/imagem sem texto extraível</x:v>
@@ -17603,7 +17629,7 @@
     </x:row>
     <x:row r="219">
       <x:c r="A219" s="24" t="str">
-        <x:v>UNA-SUS-UFMA_Saúde Digital Noções fundamentais_Certificado.pdf</x:v>
+        <x:v>UNA-SUS_UFMA_Etica e Responsabilidade_Saude Digital_Certificado Extensão.pdf</x:v>
       </x:c>
       <x:c r="B219" s="24" t="str">
         <x:v>PDF/imagem sem texto extraível</x:v>
@@ -17618,7 +17644,7 @@
     </x:row>
     <x:row r="220">
       <x:c r="A220" s="24" t="str">
-        <x:v>UNA-SUS-UFMA_Transf Digital_Extensao_Certificado.pdf</x:v>
+        <x:v>UNA-SUS_UFMA_Programa_Aperfeicoamento_Saude Digital_Certificado.pdf</x:v>
       </x:c>
       <x:c r="B220" s="24" t="str">
         <x:v>PDF/imagem sem texto extraível</x:v>
@@ -17633,10 +17659,10 @@
     </x:row>
     <x:row r="221">
       <x:c r="A221" s="24" t="str">
-        <x:v>UNA-SUS_Certificado_Introducao Saúde Digital.pdf</x:v>
+        <x:v>VMEdu_SFC_PedroLamounierSampaio-1182483.pdf</x:v>
       </x:c>
       <x:c r="B221" s="24" t="str">
-        <x:v>PDF/imagem sem texto extraível</x:v>
+        <x:v>Carga horária não localizada</x:v>
       </x:c>
       <x:c r="C221" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
@@ -17648,76 +17674,16 @@
     </x:row>
     <x:row r="222">
       <x:c r="A222" s="24" t="str">
-        <x:v>UNA-SUS_UFMA_Cultura da Saúde Digital_Certificado de Extensão_.pdf</x:v>
+        <x:v>Your D-U-N-S Number is enclosed_.pdf</x:v>
       </x:c>
       <x:c r="B222" s="24" t="str">
-        <x:v>PDF/imagem sem texto extraível</x:v>
+        <x:v>Carga horária não localizada</x:v>
       </x:c>
       <x:c r="C222" s="24" t="str">
         <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
       </x:c>
       <x:c r="D222" s="24" t="str"/>
       <x:c r="E222" s="24" t="str">
-        <x:v>Pendente</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="223">
-      <x:c r="A223" s="24" t="str">
-        <x:v>UNA-SUS_UFMA_Etica e Responsabilidade_Saude Digital_Certificado Extensão.pdf</x:v>
-      </x:c>
-      <x:c r="B223" s="24" t="str">
-        <x:v>PDF/imagem sem texto extraível</x:v>
-      </x:c>
-      <x:c r="C223" s="24" t="str">
-        <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
-      </x:c>
-      <x:c r="D223" s="24" t="str"/>
-      <x:c r="E223" s="24" t="str">
-        <x:v>Pendente</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="224">
-      <x:c r="A224" s="24" t="str">
-        <x:v>UNA-SUS_UFMA_Programa_Aperfeicoamento_Saude Digital_Certificado.pdf</x:v>
-      </x:c>
-      <x:c r="B224" s="24" t="str">
-        <x:v>PDF/imagem sem texto extraível</x:v>
-      </x:c>
-      <x:c r="C224" s="24" t="str">
-        <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
-      </x:c>
-      <x:c r="D224" s="24" t="str"/>
-      <x:c r="E224" s="24" t="str">
-        <x:v>Pendente</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="225">
-      <x:c r="A225" s="24" t="str">
-        <x:v>VMEdu_SFC_PedroLamounierSampaio-1182483.pdf</x:v>
-      </x:c>
-      <x:c r="B225" s="24" t="str">
-        <x:v>Carga horária não localizada</x:v>
-      </x:c>
-      <x:c r="C225" s="24" t="str">
-        <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
-      </x:c>
-      <x:c r="D225" s="24" t="str"/>
-      <x:c r="E225" s="24" t="str">
-        <x:v>Pendente</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="226">
-      <x:c r="A226" s="24" t="str">
-        <x:v>Your D-U-N-S Number is enclosed_.pdf</x:v>
-      </x:c>
-      <x:c r="B226" s="24" t="str">
-        <x:v>Carga horária não localizada</x:v>
-      </x:c>
-      <x:c r="C226" s="24" t="str">
-        <x:v>Conferir visualmente e, no Coursera, abrir o link de verificação do certificado</x:v>
-      </x:c>
-      <x:c r="D226" s="24" t="str"/>
-      <x:c r="E226" s="24" t="str">
         <x:v>Pendente</x:v>
       </x:c>
     </x:row>

</xml_diff>